<commit_message>
Haven verplaatst naar de vastgestelde locatie Porto Central, Presidente Kennedy (ES)
Havenas (A1) nu door het bouwterrein fase 1 aan het strand,
E 297.135 / N 7.650.000, azimut 110 graden haaks op de kust.
SO, DO, PDF-bladen, maatstaat, rekenboek, toelichting en webkaart
opnieuw gegenereerd; teksten over de locatiekeuze aangepast.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -1497,16 +1497,16 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>296650</v>
+        <v>297135</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7648300</v>
+        <v>7650000</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-21.2556262</v>
+        <v>-21.2403293</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-40.9597006</v>
+        <v>-40.9548262</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>0</v>
@@ -1527,16 +1527,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297090.17</v>
+        <v>297557.86</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7648206.44</v>
+        <v>7649846.09</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2565204</v>
+        <v>-21.2417663</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9554718</v>
+        <v>-40.9507715</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>450</v>
@@ -1557,16 +1557,16 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>298753.02</v>
+        <v>299155.34</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7647852.99</v>
+        <v>7649264.66</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2598972</v>
+        <v>-21.2471941</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9394954</v>
+        <v>-40.9354532</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>2150</v>
@@ -1587,16 +1587,16 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300220.24</v>
+        <v>300564.88</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7647541.12</v>
+        <v>7648751.63</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2628755</v>
+        <v>-21.2519822</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9253979</v>
+        <v>-40.921936</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>3650</v>
@@ -1617,16 +1617,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308534.49</v>
+        <v>308552.27</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7645773.87</v>
+        <v>7645844.46</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2797312</v>
+        <v>-21.2790957</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8454996</v>
+        <v>-40.8453204</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>12150</v>
@@ -1647,16 +1647,16 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>296871.99</v>
+        <v>297540.35</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>7649632.97</v>
+        <v>7651289.11</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-21.2436142</v>
+        <v>-21.2287338</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-40.9574032</v>
+        <v>-40.9507688</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>-60</v>
@@ -1677,16 +1677,16 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>296248.26</v>
+        <v>296514.29</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>7646698.53</v>
+        <v>7648470.03</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-21.2700425</v>
+        <v>-21.2540757</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-40.9637624</v>
+        <v>-40.9609876</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>-60</v>
@@ -1707,16 +1707,16 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>296158.8</v>
+        <v>296695.12</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7648634.43</v>
+        <v>7650399.54</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-21.2525512</v>
+        <v>-21.2366723</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-40.9643922</v>
+        <v>-40.9590153</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>-550</v>
@@ -1737,16 +1737,16 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>294593.76</v>
+        <v>295191.62</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7648967.09</v>
+        <v>7650946.77</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-21.2493709</v>
+        <v>-21.2315619</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-40.9794274</v>
+        <v>-40.9734306</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>-2150</v>
@@ -1767,16 +1767,16 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>297253.57</v>
+        <v>297545.53</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7646955.12</v>
+        <v>7648584.21</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-21.2678381</v>
+        <v>-21.2531599</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-40.9540468</v>
+        <v>-40.9510404</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>870</v>
@@ -1797,16 +1797,16 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>294351.35</v>
+        <v>294926.72</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7648788.59</v>
+        <v>7650803.75</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-21.2509553</v>
+        <v>-21.2328236</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-40.9817839</v>
+        <v>-40.9759991</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>-2350</v>
@@ -1818,14 +1818,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lokaal havenstelsel: oorsprong A1; u-as azimut 102 gr (zeewaarts), v-as azimut 12 gr (langs de kust).</t>
+          <t>Lokaal havenstelsel: oorsprong A1; u-as azimut 110 gr (zeewaarts), v-as azimut 20 gr (langs de kust).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E = 296650,0 + u*sin(102 gr) + v*sin(12 gr);  N = 7648300,0 + u*cos(102 gr) + v*cos(12 gr).</t>
+          <t>E = 297135.0 + u*sin(110 gr) + v*sin(20 gr);  N = 7650000.0 + u*cos(110 gr) + v*cos(20 gr).</t>
         </is>
       </c>
     </row>
@@ -1916,16 +1916,16 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>296650</v>
+        <v>297135</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7648300</v>
+        <v>7650000</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-21.2556262</v>
+        <v>-21.2403293</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-40.9597006</v>
+        <v>-40.9548262</v>
       </c>
     </row>
     <row r="6">
@@ -1940,16 +1940,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>296796.72</v>
+        <v>297275.95</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7648268.81</v>
+        <v>7649948.7</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2559243</v>
+        <v>-21.2408083</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.958291</v>
+        <v>-40.9534746</v>
       </c>
     </row>
     <row r="7">
@@ -1964,16 +1964,16 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>298410.67</v>
+        <v>298826.45</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7647925.76</v>
+        <v>7649384.36</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2592021</v>
+        <v>-21.2460767</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9427847</v>
+        <v>-40.938607</v>
       </c>
     </row>
     <row r="8">
@@ -1988,16 +1988,16 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300562.59</v>
+        <v>300893.77</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7647468.35</v>
+        <v>7648631.92</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2635703</v>
+        <v>-21.2530993</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9221084</v>
+        <v>-40.9187818</v>
       </c>
     </row>
     <row r="9">
@@ -2012,16 +2012,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308551.63</v>
+        <v>308863.33</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7647887.04</v>
+        <v>7647934.67</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2606497</v>
+        <v>-21.2602524</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8450966</v>
+        <v>-40.8420884</v>
       </c>
     </row>
   </sheetData>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hoek bouwterrein N 7.650 km</t>
+          <t>Hoek bouwterrein fase 1 aan het strand</t>
         </is>
       </c>
       <c r="C19" s="9" t="n"/>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Havenas haaks op de kust (azimut 102 gr), kustpunt A1 E 296.650,0 / N 7.648.300,0; tussen kustbebouwing (zuid, N ca. 7.646.300) en zichtbaar grondwerk (noord, N ca. 7.650.000); rivier en wetland in het zuidwesten vermeden.</t>
+          <t>Locatie vastgesteld: Porto Central, Presidente Kennedy - Espírito Santo (29350-000). Havenas haaks op de kust (azimut 110 gr) door het bouwterrein fase 1; kustpunt A1 E 297.135,0 / N 7.650.000,0; bekkens landinwaarts op het Porto Central-terrein.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Eigendom/bestemming en relatie met het werkelijke Porto Central-terrein bij de begeleider navragen.</t>
+          <t>Ligging van de havenas op het terrein afstemmen met het bouwterrein fase 1 / masterplan.</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>SO: LNG aan de noordzijde; wortel noorddam en tanks bij grondwerk N 7.650 km en tegen de containeruitbreiding.</t>
+          <t>SO: LNG aan de noordzijde; tanks direct tegen de containeruitbreiding en de hoofdcorridor, LNG-schepen langs de containerkade.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">

</xml_diff>

<commit_message>
SO en DO hertekend naar de vorm van het Porto Central-masterplan
- Gebogen noord- en zuiddam met ingang naar het OZO, containervinger met
  1.600 m kade aan de voorhaven, hoofdbekken met graan aan de noordkade,
  insteekbekken met RoRo op de tweede vinger, tank- en energiezone langs
  de zuidrand en LNG-steiger achter de zuidelijke dam
- Nieuwe bespreekpunten SO, besluitenlijst en vergelijking met het
  masterplan; masterplan als vormreferentie op de bladen
- LandXML voor Civil 3D: geulas (Alignment) en ontwerpbodem (TIN)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>687</v>
+        <v>87</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>281</v>
+        <v>140</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>762</v>
+        <v>939</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
@@ -1138,33 +1138,29 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>LNG-zone (tanks + hervergassing)</t>
+          <t>LNG-tanks tot containerterrein</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>25</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>465</v>
       </c>
       <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Invoer D51-D52</t>
-        </is>
-      </c>
+      <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>3 tanks + optie 4e</t>
+          <t>QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Centrale + utilities (reservering)</t>
+          <t>LNG-zone (tanks + hervergassing)</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1173,24 +1169,24 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>49.5</v>
+        <v>30</v>
       </c>
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>geen vast oppervlak</t>
+          <t>Invoer D51-D52</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>3 tanks + optie 4e</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Havendiensten / sleepboten</t>
+          <t>Centrale + utilities (reservering)</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1199,10 +1195,14 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>29.4</v>
+        <v>52.5</v>
       </c>
       <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>geen vast oppervlak</t>
+        </is>
+      </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
           <t>reservering</t>
@@ -1212,7 +1212,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Reserveterreinen</t>
+          <t>Havendiensten / sleepboten</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>161.1</v>
+        <v>15.4</v>
       </c>
       <c r="D30" s="3" t="n"/>
       <c r="E30" s="3" t="inlineStr"/>
@@ -1234,49 +1234,53 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte binnenbekken (schepen aan beide zijden)</t>
+          <t>Reserveterreinen</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>354</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>220</v>
-      </c>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>237.8</v>
+      </c>
+      <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>reservering</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>Vrije breedte insteekbekken met RoRo-schip</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>720000</v>
-      </c>
-      <c r="D32" s="3" t="n"/>
+        <v>407</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>220</v>
+      </c>
       <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Binnenbekken gebaggerd fase 1</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1285,7 +1289,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>810000</v>
+        <v>1842500</v>
       </c>
       <c r="D33" s="3" t="n"/>
       <c r="E33" s="3" t="inlineStr"/>
@@ -1294,7 +1298,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1303,7 +1307,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1057500</v>
+        <v>2102500</v>
       </c>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1312,7 +1316,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1321,7 +1325,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1134585</v>
+        <v>2362500</v>
       </c>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="inlineStr"/>
@@ -1330,7 +1334,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1339,24 +1343,16 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2192085</v>
+        <v>760465</v>
       </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C6</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>ingevuld</t>
-        </is>
-      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Havenbekken totaal (zone 1)</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1365,24 +1361,24 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2200000</v>
+        <v>3122965</v>
       </c>
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk C7 + C8</t>
+          <t>Grondwerk C6</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>splitsing open</t>
+          <t>ingevuld</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1391,15 +1387,41 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>3079000</v>
+        <v>2200000</v>
       </c>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>Grondwerk C7 + C8</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>splitsing open</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>3019000</v>
+      </c>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
           <t>Grondwerk D21</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>
@@ -1416,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1527,22 +1549,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297557.86</v>
+        <v>297451.11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7649846.09</v>
+        <v>7649991.36</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2417663</v>
+        <v>-21.2404426</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9507715</v>
+        <v>-40.9517825</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -1557,22 +1579,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>299155.34</v>
+        <v>298876.85</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7649264.66</v>
+        <v>7649065.48</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2471941</v>
+        <v>-21.2489619</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9354532</v>
+        <v>-40.9381592</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>2150</v>
+        <v>1956.4</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0</v>
+        <v>-282.4</v>
       </c>
     </row>
     <row r="8">
@@ -1587,22 +1609,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300564.88</v>
+        <v>300134.86</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7648751.63</v>
+        <v>7648248.52</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2519822</v>
+        <v>-21.2564782</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.921936</v>
+        <v>-40.9261374</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3650</v>
+        <v>3418</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0</v>
+        <v>-619.8</v>
       </c>
     </row>
     <row r="9">
@@ -1617,22 +1639,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308552.27</v>
+        <v>307263.56</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7645844.46</v>
+        <v>7643619.09</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2790957</v>
+        <v>-21.2990555</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8453204</v>
+        <v>-40.8579896</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>12150</v>
+        <v>11700.1</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0</v>
+        <v>-2531.9</v>
       </c>
     </row>
     <row r="10">
@@ -1647,22 +1669,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>297540.35</v>
+        <v>297737.85</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>7651289.11</v>
+        <v>7651802.52</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-21.2287338</v>
+        <v>-21.2241196</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-40.9507688</v>
+        <v>-40.9488056</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-60</v>
+        <v>-50</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1350</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="11">
@@ -1677,22 +1699,22 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>296514.29</v>
+        <v>296314.32</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>7648470.03</v>
+        <v>7648329.97</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-21.2540757</v>
+        <v>-21.255318</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-40.9609876</v>
+        <v>-40.9629306</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-60</v>
+        <v>-200</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>-1650</v>
+        <v>-1850</v>
       </c>
     </row>
     <row r="12">
@@ -1703,26 +1725,26 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Containerkade begin (F1)</t>
+          <t>Containerkade noordeinde (F1)</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>296695.12</v>
+        <v>297135.17</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7650399.54</v>
+        <v>7650585.23</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-21.2366723</v>
+        <v>-21.2350446</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-40.9590153</v>
+        <v>-40.9547548</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-550</v>
+        <v>-200</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>225</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13">
@@ -1733,26 +1755,26 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Containerkade eind (F3)</t>
+          <t>Containerkade zuideinde (F3)</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>295191.62</v>
+        <v>296587.94</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7650946.77</v>
+        <v>7649081.73</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-21.2315619</v>
+        <v>-21.2485603</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-40.9734306</v>
+        <v>-40.960205</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-2150</v>
+        <v>-200</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>225</v>
+        <v>-1050</v>
       </c>
     </row>
     <row r="14">
@@ -1767,22 +1789,22 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>297545.53</v>
+        <v>297377.21</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7648584.21</v>
+        <v>7648560.34</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-21.2531599</v>
+        <v>-21.2533567</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-40.9510404</v>
+        <v>-40.9526645</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>870</v>
+        <v>720</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>-1190</v>
+        <v>-1270</v>
       </c>
     </row>
     <row r="15">
@@ -1793,44 +1815,74 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Eind binnenbekken</t>
+          <t>Graankade midden</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>294926.72</v>
+        <v>296729.58</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7650803.75</v>
+        <v>7651371.36</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-21.2328236</v>
+        <v>-21.2279005</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-40.9759991</v>
+        <v>-40.9585675</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-2350</v>
+        <v>-850</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Lokaal havenstelsel: oorsprong A1; u-as azimut 110 gr (zeewaarts), v-as azimut 20 gr (langs de kust).</t>
-        </is>
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>RoRo-kade midden</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>295815.28</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>7650906.01</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>-21.2320002</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>-40.9674288</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>-1550</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E = 297135.0 + u*sin(110 gr) + v*sin(20 gr);  N = 7650000.0 + u*cos(110 gr) + v*cos(20 gr).</t>
+          <t>Lokaal havenstelsel: oorsprong A1; u-as azimut 110 gr (zeewaarts), v-as azimut 20 gr (langs de kust).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>E = 297135.0 + u*sin(110 gr) + v*sin(20 gr);  N = 7650000.0 + u*cos(110 gr) + v*cos(20 gr).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Lat/lon via pyproj (EPSG:31984 -&gt; EPSG:4326).</t>
         </is>
@@ -1912,7 +1964,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Kustpunt havenas</t>
+          <t>Kustpunt havenas (waterlijn)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1936,20 +1988,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Middelpunt draaikom</t>
+          <t>Middelpunt vrije draaikom</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297275.95</v>
+        <v>297263.17</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7649948.7</v>
+        <v>7650059.77</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2408083</v>
+        <v>-21.2398039</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9534746</v>
+        <v>-40.9535845</v>
       </c>
     </row>
     <row r="7">
@@ -1964,16 +2016,16 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>298826.45</v>
+        <v>298646.98</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7649384.36</v>
+        <v>7649161.11</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2460767</v>
+        <v>-21.2480728</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.938607</v>
+        <v>-40.9403621</v>
       </c>
     </row>
     <row r="8">
@@ -1988,16 +2040,16 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300893.77</v>
+        <v>300492.05</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7648631.92</v>
+        <v>7647962.91</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2530993</v>
+        <v>-21.2590966</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9187818</v>
+        <v>-40.9227299</v>
       </c>
     </row>
     <row r="9">
@@ -2012,16 +2064,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308863.33</v>
+        <v>308100.51</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7647934.67</v>
+        <v>7645490.77</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2602524</v>
+        <v>-21.2822419</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8420884</v>
+        <v>-40.8497131</v>
       </c>
     </row>
   </sheetData>
@@ -2700,27 +2752,27 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Havenmond</t>
+          <t>Havenvorm</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>SO: 350 m tussen damhartlijnen, vrij tussen footprints maar 260 m.</t>
+          <t>SO: eerste schets naar het Porto Central-masterplan.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>DO: dammen verlegd, 350 m vrij tussen de golfbrekerfootprints (90 m breed).</t>
+          <t>DO: vorm van het masterplan aangehouden: twee gebogen dammen met ingang naar het OZO (11/14), hoofdbekken langs de noordzijde met graan aan de noordkade (10), containervinger met kade aan de voorhaven (6), insteekbekken en tweede vinger (7/8), tank- en energiezone langs de zuidrand (9) en LNG-steiger bij de zuidelijke dam (18). Maten volgen het rekenboek, niet het masterplan.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Verwerkt</t>
+          <t>Vastgelegd</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Na golfbrekerontwerp (kruin, taluds) footprint en vrije breedte opnieuw meten.</t>
+          <t>Masterplan-functies buiten het groepsprogramma (erts, olie, werf) als reserve aangeduid.</t>
         </is>
       </c>
     </row>
@@ -2732,17 +2784,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Draaikom en stopweg</t>
+          <t>Havenmond</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>SO: middelpunt 150 m uit de kust; draaikom raakt landhoeken (1,6 ha); stopweg 1.650 m &lt; 5 LOA (1.670 m).</t>
+          <t>SO: 350 m tussen damhartlijnen, vrij tussen de footprints maar 260 m.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>DO: middelpunt 450 m uit de kust, mond op 2.150 m: stopweg 1.700 m = 5,1 LOA; draaikom 687 m vrij van afgemeerde schepen en 281 m van kades/dammen.</t>
+          <t>DO: dammen verlegd, 350 m vrij tussen de golfbrekerfootprints (90 m breed).</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2752,7 +2804,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Nautische (simulator)toets met sleepboten.</t>
+          <t>Na golfbrekerontwerp (kruin, taluds) footprint en vrije breedte opnieuw meten.</t>
         </is>
       </c>
     </row>
@@ -2764,27 +2816,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Toegangsgeul</t>
+          <t>Draaikom en stopweg</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>SO: knik van 15 gr op 2,2 km buiten de mond.</t>
+          <t>SO: draaikom overlapt ligplaats C1 en de containerkade (2,0 ha); stopweg 1.650 m &lt; 5 LOA (1.670 m).</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: rechte geul, 220 m bodembreedte, -18,20 m MLWS, as in het verlengde van de havenas. Lengte buiten de mond voorlopig 10.000 m.</t>
+          <t>DO: draaikom 200 m zeewaarts verschoven, mond verder uit de kust: stopweg 1.700 m = 5,1 LOA; draaikom 87 m vrij van afgemeerde schepen en 140 m van kades/dammen.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Deels open</t>
+          <t>Verwerkt</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Eindpunt op de -18,2 m MLWS-dieptelijn van de bathymetrische kaart leggen; MLWS-DHN koppelen; geullengte terugzetten in Nautiek D31.</t>
+          <t>Nautische (simulator)toets met sleepboten; containerschepen varen na het draaien achteruit of met sleepboten naar C2-C4.</t>
         </is>
       </c>
     </row>
@@ -2796,27 +2848,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sleepbootkoppelpunt</t>
+          <t>Toegangsgeul en sleepboten</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>SO: niet getekend.</t>
+          <t>SO: geul knikt 15 gr op 2,2 km buiten de mond; geen sleepbootkoppelpunt.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>DO: koppelpunt op de geulas, 1.500 m buiten de mond (A4).</t>
+          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Lengte buiten de mond voorlopig 10.000 m.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Verwerkt</t>
+          <t>Deels open</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Bevestigen met loods/sleepdienst en golfklimaat (werkbaarheid).</t>
+          <t>Eindpunt op de -18,2 m MLWS-dieptelijn van de bathymetrie leggen; MLWS-DHN koppelen; geullengte terugzetten in Nautiek D31.</t>
         </is>
       </c>
     </row>
@@ -2833,12 +2885,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>SO: LNG aan de noordzijde; tanks direct tegen de containeruitbreiding en de hoofdcorridor, LNG-schepen langs de containerkade.</t>
+          <t>SO: LNG-zone direct achter het containerterrein; tanks op 105 m.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DO: LNG-steiger aan de lijzijde van de zuidelijke dam in eigen insteek, 762 m vrij van de draaikom; tankzone 25 ha met 3 x 180.000 m3 en ruimte voor een 4e tank; 291 m tot RoRo-terrein.</t>
+          <t>DO: tank- en energiezone verschoven naar de zuidrand (masterplan 9); tanks op 465 m van het containerterrein, weg-/spoorcorridor ertussen; LNG-ligplaats 939 m vrij van de draaikom; ruimte voor een 4e tank.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -2865,12 +2917,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>SO: gedeeld perceel, weg kruist het terrein.</t>
+          <t>SO: gedeeld perceel van 66 ha aan de noordkade, weg kruist het terrein.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DO: ieder 30 ha (500 x 600 m) met eigen kade van 300 m, eigen inrit; weg en spoor achter de percelen.</t>
+          <t>DO: graan 30 ha aan de noordkade (masterplan 10) met silo en transportband; RoRo 30 ha op de tweede vinger aan het insteekbekken (masterplan 7/8), ieder een eigen kade van 300 m en eigen inrit.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -2897,12 +2949,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>SO: containerfase 1 aan het landeinde, heel bekken in fase 1 baggeren.</t>
+          <t>SO: containerfase 1 aan het zuideinde van de vinger; alle bekkens in fase 1 baggeren.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: fase 1 bij de ingang; binnenbekken in drie stappen (72,0 / 81,0 / 105,8 ha); uitbreiding aan het doodlopende eind, geen vaarwegblokkade.</t>
+          <t>DO: fase 1 bij de ingang (C1-C2), kade groeit zuidwaarts; bekkens gebaggerd 184,2 / 210,2 / 236,2 ha; reserve-insteek en hoofdbekken-west (96,8 ha) pas in fase 4.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -2929,12 +2981,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>SO: centrale achter de LNG-tanks aan de noordzijde.</t>
+          <t>SO: centrale naast de LNG-zone, tegen het containerterrein.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>DO: reservering 49,5 ha naast de LNG-zone; koelwaterinlaat in de voorhaven en uitlaat buiten de zuidelijke dam (indicatief).</t>
+          <t>DO: reservering 52,5 ha in de zuidelijke energiezone; gasleiding naar het regionale net; koelwaterinlaat in de voorhaven, uitlaat buiten de zuidelijke dam (indicatief).</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -2961,12 +3013,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>SO: corridor aan de westzijde, weg door terminalperceel.</t>
+          <t>SO: corridor aan de westzijde, weg door het graan/RoRo-perceel.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>DO: hoofdweg + spoor in corridor aan de westzijde, takken achter de terminalpercelen met aparte poorten.</t>
+          <t>DO: hoofdweg + spoor aan de westzijde (zoals de ringweg in het masterplan), takken achter de percelen: noord (graan), midden (RoRo), zuid (containers, LNG, centrale); aparte poorten.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -3030,7 +3082,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken 2.192.085 m2, geul buiten de mond 2.200.000 m2, terreinophoging 3.079.000 m2 ingevuld.</t>
+          <t>Havenbekken 3.122.965 m2, geul buiten de mond 2.200.000 m2, terreinophoging 3.019.000 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -3040,7 +3092,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Bestaande diepten/hoogten uit bathymetrie en hoogtemodel invoeren; geul splitsen op DHN -15 m.</t>
+          <t>Bathymetrie als Civil 3D-oppervlak inlezen en volume tegen Ontwerpbodem_DO berekenen; geul splitsen op DHN -15 m.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DO overgetrokken van de Porto Central-render
- Definitief ontwerp volgt de render: gebogen dammen, hoofdbekken
  oost-west, schuine vingers en insteekbekkens evenwijdig aan de kust,
  containervinger met kraankade aan de insteek, tankpark langs de
  zuidrand en LNG-steiger bij de zuidelijke dam
- Render op schaal (10,035 m/px) en op de kust gedraaid; in de DXF als
  overtrek-laag HV-REFERENTIE en in de PDF als blad DO-05
- DO-bladen op 1:15.000 / 1:30.000; teksten, besluitenlijst en
  maatstaat bijgewerkt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>11700</v>
+        <v>11727</v>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="inlineStr">
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>87</v>
+        <v>646</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1700</v>
+        <v>1727</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>1670</v>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>800</v>
+        <v>802.1921820131856</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>800</v>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1200</v>
+        <v>1203.288273019332</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>1200</v>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1600</v>
+        <v>1604.384364026371</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>1600</v>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>30</v>
+        <v>30.4</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>30</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>30</v>
+        <v>30.2</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>30</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>939</v>
+        <v>729</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>465</v>
+        <v>296</v>
       </c>
       <c r="D27" s="3" t="n"/>
       <c r="E27" s="3" t="inlineStr"/>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>30</v>
+        <v>31.9</v>
       </c>
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="inlineStr">
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>52.5</v>
+        <v>47.1</v>
       </c>
       <c r="D29" s="3" t="n"/>
       <c r="E29" s="3" t="inlineStr">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>15.4</v>
+        <v>43</v>
       </c>
       <c r="D30" s="3" t="n"/>
       <c r="E30" s="3" t="inlineStr"/>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>237.8</v>
+        <v>850.2</v>
       </c>
       <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="inlineStr"/>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>407</v>
+        <v>479</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>220</v>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1842500</v>
+        <v>1138629</v>
       </c>
       <c r="D33" s="3" t="n"/>
       <c r="E33" s="3" t="inlineStr"/>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2102500</v>
+        <v>1369033</v>
       </c>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>2362500</v>
+        <v>1599438</v>
       </c>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="inlineStr"/>
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>760465</v>
+        <v>1049760</v>
       </c>
       <c r="D36" s="3" t="n"/>
       <c r="E36" s="3" t="inlineStr"/>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>3122965</v>
+        <v>2649198</v>
       </c>
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="inlineStr">
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>3019000</v>
+        <v>3266194</v>
       </c>
       <c r="D39" s="3" t="n"/>
       <c r="E39" s="3" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>u lokaal (m)</t>
+          <t>x render (px)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>v lokaal (m)</t>
+          <t>y render (px)</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Kustpunt havenas (waterlijn)</t>
+          <t>Referentiepunt kust (render 812,5 / 275)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1531,10 +1531,10 @@
         <v>-40.9548262</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0</v>
+        <v>812.5</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6">
@@ -1549,22 +1549,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297451.11</v>
+        <v>297352.65</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7649991.36</v>
+        <v>7649661.36</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2404426</v>
+        <v>-21.2434116</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9517825</v>
+        <v>-40.95277</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>300</v>
+        <v>828</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>100</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7">
@@ -1579,22 +1579,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>298876.85</v>
+        <v>299054.7</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7649065.48</v>
+        <v>7649370.46</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2489619</v>
+        <v>-21.2462275</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9381592</v>
+        <v>-40.9364101</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1956.4</v>
+        <v>990</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>-282.4</v>
+        <v>370</v>
       </c>
     </row>
     <row r="8">
@@ -1609,22 +1609,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300134.86</v>
+        <v>300533.26</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7648248.52</v>
+        <v>7649117.76</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2564782</v>
+        <v>-21.2486725</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9261374</v>
+        <v>-40.9221977</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3418</v>
+        <v>1130.7</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>-619.8</v>
+        <v>420.4</v>
       </c>
     </row>
     <row r="9">
@@ -1639,22 +1639,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>307263.56</v>
+        <v>308911.77</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7643619.09</v>
+        <v>7647685.81</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2990555</v>
+        <v>-21.262505</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8579896</v>
+        <v>-40.8416497</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>11700.1</v>
+        <v>1928.2</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>-2531.9</v>
+        <v>705.9</v>
       </c>
     </row>
     <row r="10">
@@ -1669,22 +1669,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>297737.85</v>
+        <v>297202.27</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>7651802.52</v>
+        <v>7650918.75</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-21.2241196</v>
+        <v>-21.2320404</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-40.9488056</v>
+        <v>-40.9540689</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-50</v>
+        <v>835</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1900</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11">
@@ -1699,22 +1699,22 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>296314.32</v>
+        <v>296285.1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>7648329.97</v>
+        <v>7647740.85</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>-21.255318</v>
+        <v>-21.2606345</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>-40.9629306</v>
+        <v>-40.9632826</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-200</v>
+        <v>690</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>-1850</v>
+        <v>482</v>
       </c>
     </row>
     <row r="12">
@@ -1729,22 +1729,22 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>297135.17</v>
+        <v>295982.49</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7650585.23</v>
+        <v>7649572.61</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-21.2350446</v>
+        <v>-21.2440597</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-40.9547548</v>
+        <v>-40.9659781</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-200</v>
+        <v>692</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>550</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13">
@@ -1759,22 +1759,22 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>296587.94</v>
+        <v>295525.07</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7649081.73</v>
+        <v>7648034.81</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-21.2485603</v>
+        <v>-21.2578946</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-40.960205</v>
+        <v>-40.9705687</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-200</v>
+        <v>620.5</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>-1050</v>
+        <v>440</v>
       </c>
     </row>
     <row r="14">
@@ -1785,26 +1785,26 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Midden LNG-ligplaats</t>
+          <t>LNG-steigerkop</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>297377.21</v>
+        <v>298268.67</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7648560.34</v>
+        <v>7648742.76</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-21.2533567</v>
+        <v>-21.2518087</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-40.9526645</v>
+        <v>-40.9440557</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>720</v>
+        <v>902</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>-1270</v>
+        <v>418</v>
       </c>
     </row>
     <row r="15">
@@ -1819,22 +1819,22 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>296729.58</v>
+        <v>296296.46</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>7651371.36</v>
+        <v>7650045.75</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-21.2279005</v>
+        <v>-21.2398224</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-40.9585675</v>
+        <v>-40.9628973</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-850</v>
+        <v>731</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>1150</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16">
@@ -1849,35 +1849,35 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>295815.28</v>
+        <v>295265.72</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7650906.01</v>
+        <v>7649177.72</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-21.2320002</v>
+        <v>-21.2475449</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-40.9674288</v>
+        <v>-40.9729295</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-1550</v>
+        <v>614.8</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>400</v>
+        <v>323.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lokaal havenstelsel: oorsprong A1; u-as azimut 110 gr (zeewaarts), v-as azimut 20 gr (langs de kust).</t>
+          <t>DO overgetrokken van de Porto Central-render: schaal 10.035 m/px, draaiing 10.0 gr, render (812,5; 275) = A1.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E = 297135.0 + u*sin(110 gr) + v*sin(20 gr);  N = 7650000.0 + u*cos(110 gr) + v*cos(20 gr).</t>
+          <t>E = 9.882546 x + 1.742559 y + 288626.228;  N = 1.742559 x + -9.882546 y + 7651301.871  (x, y = renderpixel, y omlaag).</t>
         </is>
       </c>
     </row>
@@ -2757,12 +2757,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>SO: eerste schets naar het Porto Central-masterplan.</t>
+          <t>SO: schematische eerste schets naar het Porto Central-masterplan (rechthoekig raster).</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>DO: vorm van het masterplan aangehouden: twee gebogen dammen met ingang naar het OZO (11/14), hoofdbekken langs de noordzijde met graan aan de noordkade (10), containervinger met kade aan de voorhaven (6), insteekbekken en tweede vinger (7/8), tank- en energiezone langs de zuidrand (9) en LNG-steiger bij de zuidelijke dam (18). Maten volgen het rekenboek, niet het masterplan.</t>
+          <t>DO: de Porto Central-render is op schaal overgetrokken (10,035 m per pixel, op de kust gedraaid): gebogen dammen met ingang naar het OZO, hoofdbekken oost-west langs de noordkade, schuine vingers en insteekbekkens evenwijdig aan de kust, containervinger (6) met de kraankade aan de insteekzijde, tankpark langs de zuidrand (9) en LNG-steiger bij de zuidelijke dam (18). Zie blad DO-05.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Masterplan-functies buiten het groepsprogramma (erts, olie, werf) als reserve aangeduid.</t>
+          <t>Olie- en droge-bulksteigers (4, 5), werf (3) en erts (2) vallen buiten het programma: weggelaten of reserve.</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: draaikom 200 m zeewaarts verschoven, mond verder uit de kust: stopweg 1.700 m = 5,1 LOA; draaikom 87 m vrij van afgemeerde schepen en 140 m van kades/dammen.</t>
+          <t>DO: draaikom in de voorhaven op de plaats van de -20 m-cirkel in de render; stopweg 1.727 m = 5,2 LOA; 646 m vrij van afgemeerde schepen en 230 m van kades/dammen.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Nautische (simulator)toets met sleepboten; containerschepen varen na het draaien achteruit of met sleepboten naar C2-C4.</t>
+          <t>Nautische (simulator)toets: bocht van de toegang naar het insteekbekken (ca. 115 gr) met sleepboten.</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DO: tank- en energiezone verschoven naar de zuidrand (masterplan 9); tanks op 465 m van het containerterrein, weg-/spoorcorridor ertussen; LNG-ligplaats 939 m vrij van de draaikom; ruimte voor een 4e tank.</t>
+          <t>DO: LNG-tanks in het oostelijke deel van het tankpark (masterplan 9), 296 m van het containerterrein met de ringweg ertussen; LNG-steiger (18) 729 m vrij van de draaikom; ruimte voor een 4e tank.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>QRA en veiligheidsafstanden; N-1-voorraadbeleid kiezen (4e tank of kleiner buffer).</t>
+          <t>QRA en veiligheidsafstanden (tanks tegen containerterrein); N-1-voorraadbeleid kiezen.</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DO: graan 30 ha aan de noordkade (masterplan 10) met silo en transportband; RoRo 30 ha op de tweede vinger aan het insteekbekken (masterplan 7/8), ieder een eigen kade van 300 m en eigen inrit.</t>
+          <t>DO: graan 30,4 ha aan de noordkade (masterplan 10) met silo en transportband; RoRo 30,2 ha in de noordoosthoek van vinger 7/8 aan het insteekbekken, ieder een eigen kade van 300 m en eigen poort.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: fase 1 bij de ingang (C1-C2), kade groeit zuidwaarts; bekkens gebaggerd 184,2 / 210,2 / 236,2 ha; reserve-insteek en hoofdbekken-west (96,8 ha) pas in fase 4.</t>
+          <t>DO: fase 1 aan de noordkop van de containervinger (C1-C2), kade groeit zuidwaarts het insteekbekken in; bekkens gebaggerd 113,9 / 136,9 / 159,9 ha; hoofdbekken west en tweede insteek (157,9 ha) in fase 4.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>DO: reservering 52,5 ha in de zuidelijke energiezone; gasleiding naar het regionale net; koelwaterinlaat in de voorhaven, uitlaat buiten de zuidelijke dam (indicatief).</t>
+          <t>DO: reservering 47,1 ha in de zuidelijke energiezone; gasleiding naar het regionale net; koelwaterinlaat in de voorhaven, uitlaat buiten de zuidelijke dam (indicatief).</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>DO: hoofdweg + spoor aan de westzijde (zoals de ringweg in het masterplan), takken achter de percelen: noord (graan), midden (RoRo), zuid (containers, LNG, centrale); aparte poorten.</t>
+          <t>DO: zoals de render: hoofdweg en spoor langs de noordrand, ontsluitingsweg aan de westzijde en een ringweg om de vingers langs het tankpark; containers, RoRo, LNG en centrale vanaf de ringweg, graan en havendiensten vanaf de noordweg.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken 3.122.965 m2, geul buiten de mond 2.200.000 m2, terreinophoging 3.019.000 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
+          <t>Havenbekken 2.649.198 m2, geul buiten de mond 2.200.000 m2, terreinophoging 3.266.194 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
SO ook op het nieuwe havenontwerp (render), versies SO 2.0 / DO 3.0
- Schetsontwerp is nu een grove eerste versie op de Porto Central-render
  met de bespreekpunten (mond 260 m vrij, draaikom tegen de vinger,
  geulknik, LNG-tanks tegen containerterrein, gedeeld graan/RoRo-perceel,
  containers F1 aan het zuideinde, alle bekkens in F1)
- Oude rechthoekige schets verwijderd; versienummer in titelblokken

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -1899,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Kustpunt havenas (waterlijn)</t>
+          <t>Referentiepunt kust (render 812,5 / 275)</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -1992,16 +1992,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297263.17</v>
+        <v>297063.74</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7650059.77</v>
+        <v>7649681.74</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2398039</v>
+        <v>-21.2431953</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9535845</v>
+        <v>-40.9555504</v>
       </c>
     </row>
     <row r="7">
@@ -2016,16 +2016,16 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>298646.98</v>
+        <v>299054.7</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7649161.11</v>
+        <v>7649370.46</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2480728</v>
+        <v>-21.2462275</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9403621</v>
+        <v>-40.9364101</v>
       </c>
     </row>
     <row r="8">
@@ -2040,16 +2040,16 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300492.05</v>
+        <v>301228.29</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7647962.91</v>
+        <v>7649030.63</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2590966</v>
+        <v>-21.2495355</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9227299</v>
+        <v>-40.9155129</v>
       </c>
     </row>
     <row r="9">
@@ -2064,16 +2064,184 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308100.51</v>
+        <v>309182.79</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7645490.77</v>
+        <v>7649882.67</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2822419</v>
+        <v>-21.2426943</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8497131</v>
+        <v>-40.8387924</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Wortel noordelijke golfbreker</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>297202.27</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>7650918.75</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>-21.2320404</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>-40.9540689</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Wortel zuidelijke golfbreker</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>296285.1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>7647740.85</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>-21.2606345</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>-40.9632826</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Containerkade noordeinde (F1)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>295982.49</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>7649572.61</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>-21.2440597</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>-40.9659781</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Containerkade zuideinde (F3)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>295525.07</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>7648034.81</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>-21.2578946</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>-40.9705687</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>LNG-steigerkop</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>298268.67</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>7648742.76</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>-21.2518087</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>-40.9440557</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Graankade midden</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>296296.46</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>7650045.75</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>-21.2398224</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>-40.9628973</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>RoRo-kade midden</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>296928.95</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>7650157.27</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>-21.2388861</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>-40.9567921</v>
       </c>
     </row>
   </sheetData>
@@ -2757,7 +2925,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>SO: schematische eerste schets naar het Porto Central-masterplan (rechthoekig raster).</t>
+          <t>SO: eerste, grove schets op de Porto Central-render.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -2821,7 +2989,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>SO: draaikom overlapt ligplaats C1 en de containerkade (2,0 ha); stopweg 1.650 m &lt; 5 LOA (1.670 m).</t>
+          <t>SO: draaikom te dicht bij de vinger: overlapt de containervinger (5,7 ha).</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -2885,7 +3053,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>SO: LNG-zone direct achter het containerterrein; tanks op 105 m.</t>
+          <t>SO: LNG-zone direct achter het containerterrein; tanks op 116 m.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -2917,7 +3085,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>SO: gedeeld perceel van 66 ha aan de noordkade, weg kruist het terrein.</t>
+          <t>SO: gedeeld perceel van 73 ha aan de noordkade, weg kruist het terrein.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Alleen opdrachtfuncties en manoeuvreerbaar ontwerp (SO 3.0 / DO 4.0)
- DO: containerkade aan de oostzijde van vinger 6 (direct aan de
  voorhaven); graan en RoRo naast elkaar aan de noordkade; tankpark met
  LNG en centrale langs de zuidrand; geen niet-opdrachtfuncties meer
- SO: containerkade in een insteekbekken met een bocht van ca. 63 gr
  vanuit een hoofdbekken van 370 m als belangrijkste bespreekpunt
- Bochtberekening in maatstaat en toelichting; geul voorlopig 18 km
  (afgeleid van Porto Central: ca. 26 km tot -25 m)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>11727</v>
+        <v>19720</v>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="inlineStr">
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>646</v>
+        <v>170</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1727</v>
+        <v>1720</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>1670</v>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>802.1921820131856</v>
+        <v>802.1921820132022</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>800</v>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1203.288273019332</v>
+        <v>1203.288273019349</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>1200</v>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1604.384364026371</v>
+        <v>1604.384364026388</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>1600</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>30.2</v>
+        <v>30.4</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>30</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>729</v>
+        <v>561</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>47.1</v>
+        <v>43.5</v>
       </c>
       <c r="D29" s="3" t="n"/>
       <c r="E29" s="3" t="inlineStr">
@@ -1234,53 +1234,49 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Reserveterreinen</t>
+          <t>Vrije breedte hoofdbekken met schip aan de kade</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="n">
-        <v>850.2</v>
-      </c>
-      <c r="D31" s="3" t="n"/>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>329</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>220</v>
+      </c>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte insteekbekken met RoRo-schip</t>
+          <t>Binnenbekken gebaggerd fase 1</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>479</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>220</v>
-      </c>
+        <v>869756</v>
+      </c>
+      <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>voldoet</t>
-        </is>
-      </c>
+      <c r="F32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1289,7 +1285,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1138629</v>
+        <v>1006559</v>
       </c>
       <c r="D33" s="3" t="n"/>
       <c r="E33" s="3" t="inlineStr"/>
@@ -1298,7 +1294,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1307,7 +1303,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1369033</v>
+        <v>1143362</v>
       </c>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1316,7 +1312,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1325,7 +1321,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1599438</v>
+        <v>1007981</v>
       </c>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="inlineStr"/>
@@ -1334,7 +1330,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>Havenbekken totaal (zone 1)</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1343,16 +1339,24 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1049760</v>
+        <v>2151343</v>
       </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C6</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>ingevuld</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1361,24 +1365,24 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2649198</v>
+        <v>3960000</v>
       </c>
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk C6</t>
+          <t>Grondwerk C7 + C8</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>ingevuld</t>
+          <t>splitsing open</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1387,41 +1391,15 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2200000</v>
+        <v>3232056</v>
       </c>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk C7 + C8</t>
+          <t>Grondwerk D21</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>splitsing open</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="n">
-        <v>3266194</v>
-      </c>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk D21</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>
@@ -1549,22 +1527,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297352.65</v>
+        <v>297534.6</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7649661.36</v>
+        <v>7649611.92</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2434116</v>
+        <v>-21.2438783</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.95277</v>
+        <v>-40.9510234</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>828</v>
+        <v>845</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>312</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7">
@@ -1579,22 +1557,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>299054.7</v>
+        <v>299233.15</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>7649370.46</v>
+        <v>7649340.79</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-21.2462275</v>
+        <v>-21.2465152</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-40.9364101</v>
+        <v>-40.9346946</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>990</v>
+        <v>1007</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>370</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8">
@@ -1609,22 +1587,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300533.26</v>
+        <v>300714.4</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7649117.76</v>
+        <v>7649104.35</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2486725</v>
+        <v>-21.2488135</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9221977</v>
+        <v>-40.9204543</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>1130.7</v>
+        <v>1148.3</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>420.4</v>
+        <v>424.8</v>
       </c>
     </row>
     <row r="9">
@@ -1639,22 +1617,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>308911.77</v>
+        <v>317008.13</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7647685.81</v>
+        <v>7646503.5</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.262505</v>
+        <v>-21.274017</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8416497</v>
+        <v>-40.7637753</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1928.2</v>
+        <v>2702.3</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>705.9</v>
+        <v>962</v>
       </c>
     </row>
     <row r="10">
@@ -1725,23 +1703,23 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Containerkade noordeinde (F1)</t>
+          <t>Containerkade noordeinde</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>295982.49</v>
+        <v>296970.74</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7649572.61</v>
+        <v>7649746.86</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-21.2440597</v>
+        <v>-21.2425969</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-40.9659781</v>
+        <v>-40.9564384</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>692</v>
+        <v>792</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>297</v>
@@ -1755,23 +1733,23 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Containerkade zuideinde (F3)</t>
+          <t>Containerkade zuideinde</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>295525.07</v>
+        <v>296513.33</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7648034.81</v>
+        <v>7648209.06</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-21.2578946</v>
+        <v>-21.2564321</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-40.9705687</v>
+        <v>-40.9610281</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>620.5</v>
+        <v>720.5</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>440</v>
@@ -1849,22 +1827,22 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>295265.72</v>
+        <v>295762.81</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7649177.72</v>
+        <v>7649951.65</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-21.2475449</v>
+        <v>-21.2406122</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-40.9729295</v>
+        <v>-40.9680487</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>614.8</v>
+        <v>677</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>323.4</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18">
@@ -1992,16 +1970,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>297063.74</v>
+        <v>297224.18</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7649681.74</v>
+        <v>7649638.7</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-21.2431953</v>
+        <v>-21.2436019</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-40.9555504</v>
+        <v>-40.9540102</v>
       </c>
     </row>
     <row r="7">
@@ -2040,16 +2018,16 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>301228.29</v>
+        <v>301231.45</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>7649030.63</v>
+        <v>7649051.49</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-21.2495355</v>
+        <v>-21.2493475</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>-40.9155129</v>
+        <v>-40.91548</v>
       </c>
     </row>
     <row r="9">
@@ -2064,16 +2042,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>309182.79</v>
+        <v>316924.72</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7649882.67</v>
+        <v>7650884.84</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2426943</v>
+        <v>-21.2344404</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.8387924</v>
+        <v>-40.7641076</v>
       </c>
     </row>
     <row r="10">
@@ -2132,7 +2110,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Containerkade noordeinde (F1)</t>
+          <t>Containerkade noordeinde</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -2156,7 +2134,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Containerkade zuideinde (F3)</t>
+          <t>Containerkade zuideinde</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -2920,17 +2898,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Havenvorm</t>
+          <t>Havenvorm en programma</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>SO: eerste, grove schets op de Porto Central-render.</t>
+          <t>SO: grove schets op de Porto Central-render.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>DO: de Porto Central-render is op schaal overgetrokken (10,035 m per pixel, op de kust gedraaid): gebogen dammen met ingang naar het OZO, hoofdbekken oost-west langs de noordkade, schuine vingers en insteekbekkens evenwijdig aan de kust, containervinger (6) met de kraankade aan de insteekzijde, tankpark langs de zuidrand (9) en LNG-steiger bij de zuidelijke dam (18). Zie blad DO-05.</t>
+          <t>DO: de vorm van Porto Central is aangehouden (gebogen dammen, ingang naar het OZO, hoofdbekken langs de noordkade, containervinger, tankpark langs de zuidrand), maar er staan alleen functies uit de opdracht in: containers, droge bulk (graan), voertuigen (RoRo), LNG en de centrale. Erts, werf, industrie, supply base, olie en het tweede insteekbekken zijn weggelaten.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2940,7 +2918,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Olie- en droge-bulksteigers (4, 5), werf (3) en erts (2) vallen buiten het programma: weggelaten of reserve.</t>
+          <t>Geen; eventuele latere uitbreiding apart onderbouwen.</t>
         </is>
       </c>
     </row>
@@ -2984,17 +2962,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Draaikom en stopweg</t>
+          <t>Manoeuvreren met grote schepen</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>SO: draaikom te dicht bij de vinger: overlapt de containervinger (5,7 ha).</t>
+          <t>SO: containerkade in een insteekbekken: een schip van 334 m moet 63 gr draaien vanuit een hoofdbekken van 370 m breed. Met een vuistregel voor de bochtstraal van minimaal 3 x LOA (ca. 1.000 m) past dat niet. Ook overlapt de draaikom de containervinger (1,5 ha).</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: draaikom in de voorhaven op de plaats van de -20 m-cirkel in de render; stopweg 1.727 m = 5,2 LOA; 646 m vrij van afgemeerde schepen en 230 m van kades/dammen.</t>
+          <t>DO: containerkade aan de oostzijde van de vinger, direct aan de voorhaven. Schepen zwaaien in de draaikom (D 720 m = 2,2 LOA) en verhalen zijwaarts met sleepboten naar de kade: geen bocht buiten de draaikom. Graan- en RoRo-schepen varen met een koerswijziging van 19 gr het hoofdbekken in en verlaten het achteruit of zwaaien vooraf in de draaikom. Draaikom 170 m vrij van afgemeerde schepen; stopweg 1.720 m = 5,1 LOA.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3004,7 +2982,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Nautische (simulator)toets: bocht van de toegang naar het insteekbekken (ca. 115 gr) met sleepboten.</t>
+          <t>Toetsen met bochtstralen uit PIANC WG121 en een nautische simulatie met sleepboten.</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3004,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Lengte buiten de mond voorlopig 10.000 m.</t>
+          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Lengte buiten de mond voorlopig 18.000 m: Porto Central meldt een toegang van ca. 26 km tot ca. -25 m; bij een vergelijkbare helling ligt de -18,2 m-lijn rond 18 km.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3053,12 +3031,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>SO: LNG-zone direct achter het containerterrein; tanks op 116 m.</t>
+          <t>SO: LNG-tanks direct achter het containerterrein, op 116 m.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DO: LNG-tanks in het oostelijke deel van het tankpark (masterplan 9), 296 m van het containerterrein met de ringweg ertussen; LNG-steiger (18) 729 m vrij van de draaikom; ruimte voor een 4e tank.</t>
+          <t>DO: tanks in het zuidelijke deel van de LNG-zone, 296 m van het containerterrein met de zuidweg ertussen; LNG-steiger achter de zuidelijke dam, 561 m vrij van de draaikom; ruimte voor een 4e tank.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3068,7 +3046,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>QRA en veiligheidsafstanden (tanks tegen containerterrein); N-1-voorraadbeleid kiezen.</t>
+          <t>QRA en veiligheidsafstanden; N-1-voorraadbeleid kiezen.</t>
         </is>
       </c>
     </row>
@@ -3080,17 +3058,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Graan en RoRo</t>
+          <t>Droge bulk (graan) en RoRo</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>SO: gedeeld perceel van 73 ha aan de noordkade, weg kruist het terrein.</t>
+          <t>SO: gedeeld perceel van 104 ha aan de noordkade, weg kruist het terrein.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DO: graan 30,4 ha aan de noordkade (masterplan 10) met silo en transportband; RoRo 30,2 ha in de noordoosthoek van vinger 7/8 aan het insteekbekken, ieder een eigen kade van 300 m en eigen poort.</t>
+          <t>DO: graan 30,4 ha en RoRo 30,4 ha naast elkaar aan de noordkade van het hoofdbekken, ieder een kade van 300 m, eigen poort aan de noordweg; graansilo met transportband, RoRo-ramp.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -3100,7 +3078,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Ramp- en rijcircuit RoRo en conveyorroute graan detailleren.</t>
+          <t>Rijcircuit RoRo en conveyorroute graan detailleren.</t>
         </is>
       </c>
     </row>
@@ -3117,12 +3095,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>SO: containerfase 1 aan het zuideinde van de vinger; alle bekkens in fase 1 baggeren.</t>
+          <t>SO: containerfase 1 aan het zuideinde; alle bekkens in fase 1 baggeren.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: fase 1 aan de noordkop van de containervinger (C1-C2), kade groeit zuidwaarts het insteekbekken in; bekkens gebaggerd 113,9 / 136,9 / 159,9 ha; hoofdbekken west en tweede insteek (157,9 ha) in fase 4.</t>
+          <t>DO: fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de voorhaven; gebaggerd 87,0 / 100,7 / 114,3 ha (hoofdbekken + ligplaatsstroken).</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -3132,7 +3110,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Bouwmethode uitbreiding naast werkende kade (damwand/kistdam) uitwerken.</t>
+          <t>Bouwmethode uitbreiding naast werkende kade uitwerken.</t>
         </is>
       </c>
     </row>
@@ -3149,12 +3127,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>SO: centrale naast de LNG-zone, tegen het containerterrein.</t>
+          <t>SO: centrale naast de LNG-zone.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>DO: reservering 47,1 ha in de zuidelijke energiezone; gasleiding naar het regionale net; koelwaterinlaat in de voorhaven, uitlaat buiten de zuidelijke dam (indicatief).</t>
+          <t>DO: reservering 43,5 ha naast de LNG-zone langs de zuidrand; gasleiding naar het regionale net; koelwater indicatief.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -3164,7 +3142,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Vermogen/proceskeuze vaststellen; recirculatie en temperatuur koelwater toetsen.</t>
+          <t>Vermogen/proceskeuze vaststellen; recirculatie koelwater toetsen.</t>
         </is>
       </c>
     </row>
@@ -3181,12 +3159,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>SO: corridor aan de westzijde, weg door het graan/RoRo-perceel.</t>
+          <t>SO: weg door het graan/RoRo-perceel.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>DO: zoals de render: hoofdweg en spoor langs de noordrand, ontsluitingsweg aan de westzijde en een ringweg om de vingers langs het tankpark; containers, RoRo, LNG en centrale vanaf de ringweg, graan en havendiensten vanaf de noordweg.</t>
+          <t>DO: noordweg langs graan, RoRo en havendienst; zuidweg langs containerterrein, LNG en centrale; beide aangesloten op het regionale net aan de westzijde, met spoor.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -3250,7 +3228,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken 2.649.198 m2, geul buiten de mond 2.200.000 m2, terreinophoging 3.266.194 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
+          <t>Havenbekken 2.151.343 m2, geul buiten de mond 3.960.000 m2, terreinophoging 3.232.056 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Vorm van de render terug, met manoeuvreerbare indeling (SO 4.0 / DO 5.0)
- Hoofdbekken, twee vingers en insteekbekkens weer zoals de render
- Containerkade aan de voorhavenzijde van vinger 6; draaikom binnenhaven
  D 460 m voor graan en RoRo op de -16 m-cirkel van de render
- Alleen opdrachtfuncties; overige ruimte = uitbreiding eigen terminals

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>30.4</v>
+        <v>30.2</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>30</v>
@@ -1084,7 +1084,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>LNG-ligplaatsenvelop</t>
+          <t>Draaikom binnenhaven (graan/RoRo)</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1093,26 +1093,26 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>400</v>
+        <v>460</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>400</v>
+        <v>458</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>tekenbrief</t>
+          <t>2 x LOA graan</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>dolphins indicatief</t>
+          <t>vrij getoetst</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>LNG-envelop tot draaikom</t>
+          <t xml:space="preserve">  afstand tot afgemeerde schepen</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>561</v>
+        <v>286</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
@@ -1131,14 +1131,14 @@
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>vrij; QRA volgt</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>LNG-tanks tot containerterrein</t>
+          <t>LNG-ligplaatsenvelop</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1147,72 +1147,74 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>296</v>
-      </c>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="inlineStr"/>
+        <v>400</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>tekenbrief</t>
+        </is>
+      </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>QRA volgt</t>
+          <t>dolphins indicatief</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>LNG-zone (tanks + hervergassing)</t>
+          <t>LNG-envelop tot draaikom</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Invoer D51-D52</t>
-        </is>
-      </c>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>561</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>3 tanks + optie 4e</t>
+          <t>vrij; QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Centrale + utilities (reservering)</t>
+          <t>LNG-tanks tot containerterrein</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>43.5</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>296</v>
       </c>
       <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>geen vast oppervlak</t>
-        </is>
-      </c>
+      <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Havendiensten / sleepboten</t>
+          <t>LNG-zone (tanks + hervergassing)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1221,80 +1223,96 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>43</v>
+        <v>31.9</v>
       </c>
       <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Invoer D51-D52</t>
+        </is>
+      </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>3 tanks + optie 4e</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte hoofdbekken met schip aan de kade</t>
+          <t>Centrale + utilities (reservering)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>329</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>geen vast oppervlak</t>
+        </is>
+      </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>reservering</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>Havendiensten / sleepboten</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>869756</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>43</v>
       </c>
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>reservering</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1006559</v>
-      </c>
-      <c r="D33" s="3" t="n"/>
+        <v>334</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>220</v>
+      </c>
       <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>Binnenbekken gebaggerd fase 1</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1303,7 +1321,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1143362</v>
+        <v>1324523</v>
       </c>
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="inlineStr"/>
@@ -1312,7 +1330,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1321,7 +1339,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1007981</v>
+        <v>1461326</v>
       </c>
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="inlineStr"/>
@@ -1330,7 +1348,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1339,24 +1357,16 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2151343</v>
+        <v>1598128</v>
       </c>
       <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C6</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>ingevuld</t>
-        </is>
-      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1365,24 +1375,16 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>3960000</v>
+        <v>1007981</v>
       </c>
       <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C7 + C8</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>splitsing open</t>
-        </is>
-      </c>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+          <t>Havenbekken totaal (zone 1)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1391,15 +1393,67 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>3232056</v>
+        <v>2606110</v>
       </c>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>Grondwerk C6</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ingevuld</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>3960000</v>
+      </c>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C7 + C8</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>splitsing open</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>3229941</v>
+      </c>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
           <t>Grondwerk D21</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>
@@ -1416,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1827,40 +1881,70 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>295762.81</v>
+        <v>295265.72</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7649951.65</v>
+        <v>7649177.72</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-21.2406122</v>
+        <v>-21.2475449</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-40.9680487</v>
+        <v>-40.9729295</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>677</v>
+        <v>614.8</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>DO overgetrokken van de Porto Central-render: schaal 10.035 m/px, draaiing 10.0 gr, render (812,5; 275) = A1.</t>
-        </is>
+        <v>323.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Middelpunt draaikom binnenhaven</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>295694.75</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>7649644.15</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>-21.2433813</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>-40.968741</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>665</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>285</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E = 9.882546 x + 1.742559 y + 288626.228;  N = 1.742559 x + -9.882546 y + 7651301.871  (x, y = renderpixel, y omlaag).</t>
+          <t>DO overgetrokken van de Porto Central-render: schaal 10.035 m/px, draaiing 10.0 gr, render (812,5; 275) = A1.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
+        <is>
+          <t>E = 9.882546 x + 1.742559 y + 288626.228;  N = 1.742559 x + -9.882546 y + 7651301.871  (x, y = renderpixel, y omlaag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Lat/lon via pyproj (EPSG:31984 -&gt; EPSG:4326).</t>
         </is>
@@ -2908,7 +2992,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>DO: de vorm van Porto Central is aangehouden (gebogen dammen, ingang naar het OZO, hoofdbekken langs de noordkade, containervinger, tankpark langs de zuidrand), maar er staan alleen functies uit de opdracht in: containers, droge bulk (graan), voertuigen (RoRo), LNG en de centrale. Erts, werf, industrie, supply base, olie en het tweede insteekbekken zijn weggelaten.</t>
+          <t>DO: de vorm van de render blijft: gebogen dammen, ingang naar het OZO, hoofdbekken langs de noordkade, twee schuine vingers met insteekbekkens en het tankpark langs de zuidrand. Er staan alleen functies uit de opdracht in: containers (vinger 6), droge bulk/graan (noordkade), voertuigen/RoRo (vinger 7/8), LNG en de centrale (zuidrand). Erts, werf, industrie en olie zijn weggelaten; de overige ruimte op vinger 7/8 en de tweede insteek zijn uitbreidingsruimte voor de eigen ladingstromen na 2045.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -2918,7 +3002,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Geen; eventuele latere uitbreiding apart onderbouwen.</t>
+          <t>Uitbreidingsruimte apart onderbouwen als de groei na 2045 aan de orde komt.</t>
         </is>
       </c>
     </row>
@@ -2967,12 +3051,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>SO: containerkade in een insteekbekken: een schip van 334 m moet 63 gr draaien vanuit een hoofdbekken van 370 m breed. Met een vuistregel voor de bochtstraal van minimaal 3 x LOA (ca. 1.000 m) past dat niet. Ook overlapt de draaikom de containervinger (1,5 ha).</t>
+          <t>SO: containerkade in het insteekbekken: een schip van 334 m moet 63 gr draaien vanuit een hoofdbekken van 371 m breed. Met een vuistregel voor de bochtstraal van minimaal 3 x LOA (ca. 1.000 m) past dat niet. Ook overlapt de draaikom de containervinger (1,5 ha) en is er binnen geen draairuimte voor graan- en RoRo-schepen.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: containerkade aan de oostzijde van de vinger, direct aan de voorhaven. Schepen zwaaien in de draaikom (D 720 m = 2,2 LOA) en verhalen zijwaarts met sleepboten naar de kade: geen bocht buiten de draaikom. Graan- en RoRo-schepen varen met een koerswijziging van 19 gr het hoofdbekken in en verlaten het achteruit of zwaaien vooraf in de draaikom. Draaikom 170 m vrij van afgemeerde schepen; stopweg 1.720 m = 5,1 LOA.</t>
+          <t>DO: containerkade aan de voorhavenzijde van vinger 6: containerschepen zwaaien in de draaikom (D 720 m = 2,2 LOA) en verhalen zijwaarts met sleepboten naar de kade, zonder bocht buiten de draaikom. Graan- en RoRo-schepen (ca. 230 m) varen met 19 gr koerswijziging het hoofdbekken in en zwaaien in een draaikom binnenhaven van D 460 m (2 x LOA) op de kruising met het insteekbekken, op de plaats van de -16 m-cirkel in de render; die ligt 286 m vrij van afgemeerde schepen. Draaikom voorhaven 170 m vrij; stopweg 1.720 m = 5,1 LOA.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3068,7 +3152,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DO: graan 30,4 ha en RoRo 30,4 ha naast elkaar aan de noordkade van het hoofdbekken, ieder een kade van 300 m, eigen poort aan de noordweg; graansilo met transportband, RoRo-ramp.</t>
+          <t>DO: graan 30,4 ha aan de noordkade (render 10) met silo en transportband; RoRo 30,2 ha in de noordoosthoek van vinger 7/8 met kade aan het insteekbekken; ieder een kade van 300 m en een eigen poort.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -3100,7 +3184,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de voorhaven; gebaggerd 87,0 / 100,7 / 114,3 ha (hoofdbekken + ligplaatsstroken).</t>
+          <t>DO: containers fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de voorhaven; gebaggerd 132,5 / 146,1 / 159,8 ha; insteek zuid, hoofdbekken west en tweede insteek (178,8 ha) pas na 2045.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -3228,7 +3312,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken 2.151.343 m2, geul buiten de mond 3.960.000 m2, terreinophoging 3.232.056 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
+          <t>Havenbekken 2.606.110 m2, geul buiten de mond 3.960.000 m2, terreinophoging 3.229.941 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
DO 6.0: terminals in detail uitgewerkt (DO-06 t/m DO-08)
- Containerterminal: apron en kraanbaan, STS-kranen per fase (6/12/20),
  RTG-stackblokken (40.557 TEU-grondslots tegen 40.444 nodig), reefer,
  lege containers, railterminal, gate, kantoor en werkplaats
- Graan: 8 silo's (169.646 t tegen 154.100 t piek), shiploaders,
  transportband, ontvangst per weg en spoor; RoRo: parkeervakken
  (ca. 9.700 auto's tegen 7.479); havendienst met VTS en sleepdienst
- LNG: tanks in tankput, hervergassing, BOG, fakkel, laadarmen en
  dolphins; centrale: 4 STEG-eenheden, hoogspanningsstation, koelwater
- Detailbladen in de PDF en als extra layouts in de DXF

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1266,43 +1266,57 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Havendiensten / sleepboten</t>
+          <t>STS-kranen F1 / F2 / F3</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="inlineStr"/>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Containers D19-F19</t>
+        </is>
+      </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>gelijk</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
+          <t>TEU-grondslots stackzone F3 (28 m2/slot)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>334</v>
+        <v>40558</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
+        <v>40444</v>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Containers F25</t>
+        </is>
+      </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
           <t>voldoet</t>
@@ -1312,148 +1326,306 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>Stackzone bruto</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>1324523</v>
-      </c>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>113.2</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Containers F26</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Graansilo's 8 x D 30 m x 40 m</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>t</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1461326</v>
-      </c>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
+        <v>169646</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>154100</v>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F9</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>RoRo-parkeercapaciteit</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>auto's</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1598128</v>
-      </c>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
+        <v>9698</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>7479</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F15</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>Centrale STEG-eenheden</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1007981</v>
-      </c>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
+        <v>2260</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>2256</v>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F30</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>rekenvoorbeeld</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Havendiensten / sleepboten</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>2606110</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>43</v>
       </c>
       <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C6</t>
-        </is>
-      </c>
+      <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>ingevuld</t>
+          <t>reservering</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>3960000</v>
-      </c>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C7 + C8</t>
-        </is>
-      </c>
+        <v>334</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>splitsing open</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
+          <t>Binnenbekken gebaggerd fase 1</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>1324523</v>
+      </c>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>1461326</v>
+      </c>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>1598128</v>
+      </c>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>1007981</v>
+      </c>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Havenbekken totaal (zone 1)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>2606110</v>
+      </c>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C6</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>ingevuld</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>3960000</v>
+      </c>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C7 + C8</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>splitsing open</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
           <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C46" s="4" t="n">
         <v>3229941</v>
       </c>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>Grondwerk D21</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>

</xml_diff>

<commit_message>
DO 7.0: golftoets, dieptezones, bodemmodel GEBCO, LNG-veiligheidszones
- Containerkade naar de westzijde van vinger 6 (insteek) en LNG-steiger achter
  het midden van de zuidelijke dam na diffractie-golftoets (nieuw blad DO-09)
- Dieptezones per scheepstype: -18,20 / -16,20 (LNG) / -13,70 (RoRo) m MLWS,
  LandXML-oppervlak per zone
- Bodemmodel GEBCO 2026 + Copernicus DEM: geul 35 km, -15 m op 24 km, baggervolumes
  per vak met de celmethode (nieuw blad DO-10), dieptelijnen in SO en DO
- LNG: tanks oostelijk (leiding ca. 1,4 km), 250 m veiligheidszones en 500 m
  controlezone; besluiten, maatstaat, rekenboek en toelichting bijgewerkt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>18000</v>
+        <v>35000</v>
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>VOORLOPIG</t>
+          <t>GEBCO, geen peiling</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>19720</v>
+        <v>36720</v>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="inlineStr">
@@ -635,14 +635,14 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>VOORLOPIG</t>
+          <t>GEBCO, geen peiling</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Vrije draaikom diameter</t>
+          <t>Vrije draaikom voorhaven diameter</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>170</v>
+        <v>416</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>220</v>
+        <v>397</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>802.1921820132022</v>
+        <v>802.1921820131856</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>800</v>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1203.288273019349</v>
+        <v>1203.288273019332</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>1200</v>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1604.384364026388</v>
+        <v>1604.384364026371</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>1600</v>
@@ -1084,7 +1084,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Draaikom binnenhaven (graan/RoRo)</t>
+          <t>Zwaaiplaats binnenhaven (met sleepboten)</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1093,14 +1093,14 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>460</v>
+        <v>500</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>458</v>
+        <v>501</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>2 x LOA graan</t>
+          <t>1,5 x LOA container</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1112,7 +1112,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  afstand tot afgemeerde schepen</t>
+          <t xml:space="preserve">  afstand tot oever</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>286</v>
+        <v>91</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
@@ -1138,61 +1138,63 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>LNG-ligplaatsenvelop</t>
+          <t>Dieptezone LNG-vaarweg en -ligplaats</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>400</v>
+          <t>m MLWS</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>-16.2</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>400</v>
+        <v>-16.2</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>tekenbrief</t>
+          <t>diepgang 12,5 + 3,7</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>dolphins indicatief</t>
+          <t>bespaart bagger</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>LNG-envelop tot draaikom</t>
+          <t>Dieptezone RoRo-ligplaats</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>561</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
+          <t>m MLWS</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>diepgang 10,0 + 3,7</t>
+        </is>
+      </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>vrij; QRA volgt</t>
+          <t>bespaart bagger</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>LNG-tanks tot containerterrein</t>
+          <t>Golftoets containers (Hs insteek)</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1201,148 +1203,148 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>296</v>
-      </c>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="inlineStr"/>
+        <v>0.01</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>DO-09</t>
+        </is>
+      </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>QRA volgt</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>LNG-zone (tanks + hervergassing)</t>
+          <t>Golftoets graan (Hs)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="D30" s="3" t="n"/>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Invoer D51-D52</t>
+          <t>DO-09</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>3 tanks + optie 4e</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Centrale + utilities (reservering)</t>
+          <t>Golftoets RoRo (Hs)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="D31" s="3" t="n"/>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0.3</v>
+      </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>geen vast oppervlak</t>
+          <t>DO-09</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>STS-kranen F1 / F2 / F3</t>
+          <t>Golftoets LNG (Hs)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>6 / 12 / 20</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>6 / 12 / 20</t>
-        </is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Containers D19-F19</t>
+          <t>DO-09</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>gelijk</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>TEU-grondslots stackzone F3 (28 m2/slot)</t>
+          <t>LNG cryogene leiding</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>slots</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>40558</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>40444</v>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Containers F25</t>
-        </is>
-      </c>
+        <v>1353</v>
+      </c>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>ingekort</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Stackzone bruto</t>
+          <t>Schepen in LNG-zone 250 m</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="n">
-        <v>113.6</v>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>113.2</v>
+        <v>0</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Containers F26</t>
+          <t>Hong Kong LNG annex</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1354,53 +1356,49 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Graansilo's 8 x D 30 m x 40 m</t>
+          <t>Containerterrein tot tankzone 250 m</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>169646</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>154100</v>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Overige terminals F9</t>
-        </is>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>voldoet; QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>RoRo-parkeercapaciteit</t>
+          <t xml:space="preserve">  afstand tot afgemeerde schepen</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>auto's</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>9698</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>7479</v>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Overige terminals F15</t>
-        </is>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr">
         <is>
           <t>voldoet</t>
@@ -1410,57 +1408,61 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Centrale STEG-eenheden</t>
+          <t>LNG-ligplaatsenvelop</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2260</v>
+        <v>400</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>2256</v>
+        <v>400</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Overige terminals F30</t>
+          <t>tekenbrief</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>rekenvoorbeeld</t>
+          <t>dolphins indicatief</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Havendiensten / sleepboten</t>
+          <t>LNG-envelop tot draaikom</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="D38" s="3" t="n"/>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>876</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>vrij; QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
+          <t>LNG-tanks tot containerterrein</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1469,163 +1471,459 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>334</v>
-      </c>
-      <c r="D39" s="3" t="n">
-        <v>220</v>
-      </c>
+        <v>296</v>
+      </c>
+      <c r="D39" s="3" t="n"/>
       <c r="E39" s="3" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>LNG-zone (tanks + hervergassing)</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>1324523</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>36.3</v>
       </c>
       <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Invoer D51-D52</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>3 tanks + optie 4e</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Centrale + utilities (reservering)</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="n">
-        <v>1461326</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>43.5</v>
       </c>
       <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>geen vast oppervlak</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>reservering</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>STS-kranen F1 / F2 / F3</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>1598128</v>
-      </c>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr"/>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Containers D19-F19</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>gelijk</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>TEU-grondslots stackzone F3 (28 m2/slot)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1007981</v>
-      </c>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
+        <v>40558</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>40444</v>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Containers F25</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Stackzone bruto</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="n">
-        <v>2606110</v>
-      </c>
-      <c r="D44" s="3" t="n"/>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>113.2</v>
+      </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk C6</t>
+          <t>Containers F26</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>ingevuld</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Graansilo's 8 x D 30 m x 40 m</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>t</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>3960000</v>
-      </c>
-      <c r="D45" s="3" t="n"/>
+        <v>169646</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>154100</v>
+      </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk C7 + C8</t>
+          <t>Overige terminals F9</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>splitsing open</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
+          <t>RoRo-parkeercapaciteit</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>auto's</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>9698</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>7479</v>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F15</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Centrale STEG-eenheden</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>2260</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>2256</v>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F30</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>rekenvoorbeeld</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Havendiensten / sleepboten</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="D48" s="3" t="n"/>
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>reservering</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>334</v>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Binnenbekken gebaggerd fase 1</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>1189081</v>
+      </c>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>1419486</v>
+      </c>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>1649890</v>
+      </c>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>1132971</v>
+      </c>
+      <c r="D53" s="3" t="n"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Havenbekken totaal (zone 1)</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>2782861</v>
+      </c>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C6</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>ingevuld</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>7700000</v>
+      </c>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk C7 + C8</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>gesplitst op -15 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Baggervolume zone 1 / 2 / 3</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>mln m3</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>59,1 / 29,9 / 3,6</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk F6-F8</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>celmethode, indicatief</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
           <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
-        <v>3229941</v>
-      </c>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="C57" s="4" t="n">
+        <v>3273444</v>
+      </c>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>Grondwerk D21</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>
@@ -1843,22 +2141,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>317008.13</v>
+        <v>333795.61</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7646503.5</v>
+        <v>7643823.84</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.274017</v>
+        <v>-21.2998354</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.7637753</v>
+        <v>-40.602281</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>2702.3</v>
+        <v>4303.4</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>962</v>
+        <v>1515.5</v>
       </c>
     </row>
     <row r="10">
@@ -1933,19 +2231,19 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>296970.74</v>
+        <v>295982.49</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7649746.86</v>
+        <v>7649572.61</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-21.2425969</v>
+        <v>-21.2440597</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-40.9564384</v>
+        <v>-40.9659781</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>792</v>
+        <v>692</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>297</v>
@@ -1963,19 +2261,19 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>296513.33</v>
+        <v>295525.07</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7648209.06</v>
+        <v>7648034.81</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-21.2564321</v>
+        <v>-21.2578946</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-40.9610281</v>
+        <v>-40.9705687</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>720.5</v>
+        <v>620.5</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>440</v>
@@ -1993,22 +2291,22 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>298268.67</v>
+        <v>297643.11</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7648742.76</v>
+        <v>7648245.24</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-21.2518087</v>
+        <v>-21.2562317</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-40.9440557</v>
+        <v>-40.9501407</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>902</v>
+        <v>832</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>418</v>
+        <v>456</v>
       </c>
     </row>
     <row r="15">
@@ -2083,22 +2381,22 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>295694.75</v>
+        <v>295569.79</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>7649644.15</v>
+        <v>7649774.96</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-21.2433813</v>
+        <v>-21.242186</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-40.968741</v>
+        <v>-40.969929</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>665</v>
+        <v>655</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>285</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19">
@@ -2298,16 +2596,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>316924.72</v>
+        <v>334306.51</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7650884.84</v>
+        <v>7652915.45</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2344404</v>
+        <v>-21.2177682</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.7641076</v>
+        <v>-40.5964717</v>
       </c>
     </row>
     <row r="10">
@@ -3228,7 +3526,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: containerkade aan de voorhavenzijde van vinger 6: containerschepen zwaaien in de draaikom (D 720 m = 2,2 LOA) en verhalen zijwaarts met sleepboten naar de kade, zonder bocht buiten de draaikom. Graan- en RoRo-schepen (ca. 230 m) varen met 19 gr koerswijziging het hoofdbekken in en zwaaien in een draaikom binnenhaven van D 460 m (2 x LOA) op de kruising met het insteekbekken, op de plaats van de -16 m-cirkel in de render; die ligt 286 m vrij van afgemeerde schepen. Draaikom voorhaven 170 m vrij; stopweg 1.720 m = 5,1 LOA.</t>
+          <t>DO: containerkade aan de westzijde van vinger 6, in het insteekbekken. Golftoets (DO-09): aan de oostzijde (voorhaven) wordt Hs 1,66 m (grens 0,5 m), in de insteek 0,01 m. Containerschepen varen met sleepboten door de draaikom (D 720 m) het hoofdbekken in, zwaaien op de zwaaiplaats binnenhaven (D 500 m = 1,5 LOA, met sleepboten; het hoofdbekken is daar verbreed) en worden achteruit de insteek in gesleept, zodat ze met de kop naar buiten afmeren. De zwaaiplaats ligt 165 m vrij van afgemeerde schepen en 91 m van de oever. Draaikom voorhaven 416 m vrij; stopweg 1.720 m = 5,1 LOA.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3260,7 +3558,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Lengte buiten de mond voorlopig 18.000 m: Porto Central meldt een toegang van ca. 26 km tot ca. -25 m; bij een vergelijkbare helling ligt de -18,2 m-lijn rond 18 km.</t>
+          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Bodemmodel uit GEBCO 2026 + Copernicus DEM (DO-10): het kustplateau is vlak (-13 tot -17 m); de natuurlijke bodem is pas op 35.000 m overal dieper dan -18,2 m MLWS (-15 m op 24.000 m). Geul daarom 35 km lang; zone 2/3 gesplitst op de -15 m-lijn.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3270,7 +3568,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Eindpunt op de -18,2 m MLWS-dieptelijn van de bathymetrie leggen; MLWS-DHN koppelen; geullengte terugzetten in Nautiek D31.</t>
+          <t>Multibeampeiling langs het tracé; MLWS-DHN koppelen; geul eventueel gefaseerd (eerst -15,5 m, getijvenster).</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3590,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DO: tanks in het zuidelijke deel van de LNG-zone, 296 m van het containerterrein met de zuidweg ertussen; LNG-steiger achter de zuidelijke dam, 561 m vrij van de draaikom; ruimte voor een 4e tank.</t>
+          <t>DO: LNG-steiger achter het midden van de zuidelijke dam (golftoets Hs 0,90 m &lt; 1,0 m; bij de havenmond 1,08 m). Tanks oostelijk in de LNG-zone: cryogene leiding ca. 1,4 km. Veiligheidszone 250 m rond schip/steiger en rond de tanks, nautische controlezone 500 m (Hong Kong LNG-terminal; literatuur 250-750 m): geen andere schepen of gebouwen in de 250 m-zones; draaikom 626 m buiten de zone, containerterrein 46 m buiten de tankzone. Ligplaats en vaarweg -16,20 m MLWS.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3302,7 +3600,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>QRA en veiligheidsafstanden; N-1-voorraadbeleid kiezen.</t>
+          <t>QRA (plaatsgebonden en groepsrisico) en definitieve zones; N-1-voorraadbeleid kiezen.</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3654,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: containers fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de voorhaven; gebaggerd 132,5 / 146,1 / 159,8 ha; insteek zuid, hoofdbekken west en tweede insteek (178,8 ha) pas na 2045.</t>
+          <t>DO: containers fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de westzijde van vinger 6; gebaggerd 118,9 / 141,9 / 165,0 ha; insteek zuid, hoofdbekken west en tweede insteek (122,1 ha) pas na 2045.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -3484,17 +3782,17 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken 2.606.110 m2, geul buiten de mond 3.960.000 m2, terreinophoging 3.229.941 m2 ingevuld; ontwerpbodem als LandXML-oppervlak voor Civil 3D.</t>
+          <t>Celmethode (30 m) op het bodemmodel: zone 1 59,1, zone 2 29,9, zone 3 3,6 mln m3 (totaal 92,5 mln m3). Dieptezones per scheepstype (diepgang + 3,7 m): containers/graan -18,20, LNG -16,20, RoRo -13,70 m MLWS; besparing 0,75 mln m3. Ontwerpbodem per dieptezone als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Deels open</t>
+          <t>Indicatief</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Bathymetrie als Civil 3D-oppervlak inlezen en volume tegen Ontwerpbodem_DO berekenen; geul splitsen op DHN -15 m.</t>
+          <t>Na peiling herberekenen (Volumes Dashboard); grondsoorten uit boringen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DO 8.0: geul met bocht, zwaaiplaats 2 x LOA, golftoets met reflectie, LNG-tanks zuidelijk
- Geul: 2,5 km recht, bocht R 3.400 m naar 145 gr, dan recht tot natuurlijk -18,2 m
  (ca. 20 km i.p.v. 35 km; geulbagger 19,5 i.p.v. 33,5 mln m3); bodemmodel vergroot
- Variant haven 1 km verder in zee doorgerekend (ongeveer kostenneutraal, niet gekozen)
- Zwaaiplaats binnenhaven D 670 m (2 x LOA), hoofdbekken daar verbreed
- Golftoets met eerste-orde reflectie (spiegelbronnen, energiesom) over de hele
  scheepslengte; maatregelen: open graan-/havendienstkade, RoRo 400 m dieper in de
  insteek, LNG-steiger op de gunstigste plek langs de dam
- LNG-tanks zuidelijk: 250 m-zone 227 m buiten het containerterrein

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0182gWmzgJD58oEPLBbTj8Qu
</commit_message>
<xml_diff>
--- a/Maatstaat/Maatstaat_en_coordinaten.xlsx
+++ b/Maatstaat/Maatstaat_en_coordinaten.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>35000</v>
+        <v>20225</v>
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>36720</v>
+        <v>21946</v>
       </c>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="inlineStr">
@@ -670,33 +670,35 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Draaikom tot afgemeerde schepen</t>
+          <t>Geul: recht stuk / bochtstraal / richting</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>416</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
+          <t>m / m / gr</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2.500 / 3.400 / 145</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>PIANC WG121 (R &gt;= 5 LOA)</t>
+        </is>
+      </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>bocht 260 m breed</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Draaikom tot kades/dammen</t>
+          <t>Geul rechtdoor (variant)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -705,24 +707,24 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>397</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
+        <v>35000</v>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>DO-10</t>
+        </is>
+      </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>afgevallen</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Havenmond vrij tussen footprints</t>
+          <t>Draaikom tot afgemeerde schepen</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -731,16 +733,14 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>350</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>350</v>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Nautiek D29</t>
-        </is>
-      </c>
+        <v>416</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>voldoet</t>
@@ -750,7 +750,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Stopweg havenmond - draaikom</t>
+          <t>Draaikom tot kades/dammen</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -759,16 +759,14 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1720</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>1670</v>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>5 x LOA</t>
-        </is>
-      </c>
+        <v>397</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
           <t>voldoet</t>
@@ -778,7 +776,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Sleepbootkoppelpunt buiten mond</t>
+          <t>Havenmond vrij tussen footprints</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -787,24 +785,26 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D14" s="3" t="n"/>
+        <v>350</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>350</v>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>rapport 5.1</t>
+          <t>Nautiek D29</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>ingetekend</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Containerkade fase 1</t>
+          <t>Stopweg havenmond - draaikom</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -813,26 +813,26 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>802.1921820131856</v>
+        <v>1720</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>800</v>
+        <v>1670</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Containers D18</t>
+          <t>5 x LOA</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>gelijk</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Containerkade fase 2</t>
+          <t>Sleepbootkoppelpunt buiten mond</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -841,26 +841,24 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1203.288273019332</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>1200</v>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Containers E18</t>
+          <t>rapport 5.1</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>gelijk</t>
+          <t>ingetekend</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Containerkade fase 3</t>
+          <t>Containerkade fase 1</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -869,14 +867,14 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1604.384364026371</v>
+        <v>802.1921820131856</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1600</v>
+        <v>800</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Containers F18</t>
+          <t>Containers D18</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -888,23 +886,23 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Containerterrein fase 1</t>
+          <t>Containerkade fase 2</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>72</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>1203.288273019332</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>72</v>
+        <v>1200</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Invoer D20 (vraag 40,8)</t>
+          <t>Containers E18</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -916,23 +914,23 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Containerterrein fase 2</t>
+          <t>Containerkade fase 3</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>108</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1604.384364026371</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>108</v>
+        <v>1600</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Invoer E20 (vraag 67,9)</t>
+          <t>Containers F18</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -944,7 +942,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Containerterrein fase 3</t>
+          <t>Containerterrein fase 1</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -953,14 +951,14 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Invoer F20 (vraag 135,9)</t>
+          <t>Invoer D20 (vraag 40,8)</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -972,23 +970,23 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Graankade</t>
+          <t>Containerterrein fase 2</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>300</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>108</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>300</v>
+        <v>108</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>rapport 8.1</t>
+          <t>Invoer E20 (vraag 67,9)</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1000,7 +998,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Graanterrein</t>
+          <t>Containerterrein fase 3</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1009,14 +1007,14 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>30.4</v>
+        <v>144</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>30</v>
+        <v>144</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Invoer D39 (vraag 5,1)</t>
+          <t>Invoer F20 (vraag 135,9)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1028,7 +1026,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>RoRo-kade</t>
+          <t>Graankade</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1044,7 +1042,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>rapport 8.2</t>
+          <t>rapport 8.1</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1056,7 +1054,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>RoRo-terrein</t>
+          <t>Graanterrein</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1065,14 +1063,14 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>30.2</v>
+        <v>30.4</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>30</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Invoer D46 (vraag 26,9)</t>
+          <t>Invoer D39 (vraag 5,1)</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1084,7 +1082,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Zwaaiplaats binnenhaven (met sleepboten)</t>
+          <t>RoRo-kade</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1093,164 +1091,164 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>501</v>
+        <v>300</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>1,5 x LOA container</t>
+          <t>rapport 8.2</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>vrij getoetst</t>
+          <t>gelijk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  afstand tot oever</t>
+          <t>RoRo-terrein</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>91</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Invoer D46 (vraag 26,9)</t>
+        </is>
+      </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>gelijk</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Dieptezone LNG-vaarweg en -ligplaats</t>
+          <t>Zwaaiplaats binnenhaven</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>m MLWS</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>-16.2</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>670</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-16.2</v>
+        <v>668</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>diepgang 12,5 + 3,7</t>
+          <t>2 x LOA container</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>bespaart bagger</t>
+          <t>vrij getoetst</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Dieptezone RoRo-ligplaats</t>
+          <t xml:space="preserve">  afstand tot oever</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>m MLWS</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>-13.7</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>-13.7</v>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>diepgang 10,0 + 3,7</t>
-        </is>
-      </c>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>bespaart bagger</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Golftoets containers (Hs insteek)</t>
+          <t>Dieptezone LNG-vaarweg en -ligplaats</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>0.01</v>
+          <t>m MLWS</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>-16.2</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.5</v>
+        <v>-16.2</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>DO-09</t>
+          <t>diepgang 12,5 + 3,7</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>bespaart bagger</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Golftoets graan (Hs)</t>
+          <t>Dieptezone RoRo-ligplaats</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>0.73</v>
+          <t>m MLWS</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>-13.7</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1</v>
+        <v>-13.7</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>DO-09</t>
+          <t>diepgang 10,0 + 3,7</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>bespaart bagger</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Golftoets RoRo (Hs)</t>
+          <t>Golftoets containers (Hs insteek)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1259,10 +1257,10 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.03</v>
+        <v>0.24</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
@@ -1278,7 +1276,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Golftoets LNG (Hs)</t>
+          <t>Golftoets graan (Hs, open kade)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1287,7 +1285,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>1</v>
@@ -1306,7 +1304,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>LNG cryogene leiding</t>
+          <t>Golftoets RoRo (Hs)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1315,36 +1313,42 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1353</v>
-      </c>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="inlineStr"/>
+        <v>0.17</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>DO-09</t>
+        </is>
+      </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>ingekort</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Schepen in LNG-zone 250 m</t>
+          <t>Golftoets LNG (Hs)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>0</v>
+        <v>0.98</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Hong Kong LNG annex</t>
+          <t>DO-09</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1356,7 +1360,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Containerterrein tot tankzone 250 m</t>
+          <t>LNG cryogene leiding</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1365,40 +1369,38 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
+        <v>1223</v>
+      </c>
+      <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>voldoet; QRA volgt</t>
+          <t>ingekort</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  afstand tot afgemeerde schepen</t>
+          <t>Schepen in LNG-zone 250 m</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>st</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>&gt;0</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Hong Kong LNG annex</t>
+        </is>
+      </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
           <t>voldoet</t>
@@ -1408,7 +1410,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>LNG-ligplaatsenvelop</t>
+          <t>Containerterrein tot tankzone 250 m</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1417,26 +1419,24 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>400</v>
-      </c>
-      <c r="D37" s="3" t="n">
-        <v>400</v>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>tekenbrief</t>
-        </is>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>dolphins indicatief</t>
+          <t>voldoet; QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>LNG-envelop tot draaikom</t>
+          <t xml:space="preserve">  afstand tot afgemeerde schepen</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>876</v>
+        <v>115</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
@@ -1455,14 +1455,14 @@
       <c r="E38" s="3" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>vrij; QRA volgt</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>LNG-tanks tot containerterrein</t>
+          <t>LNG-ligplaatsenvelop</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1471,176 +1471,174 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>296</v>
-      </c>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="inlineStr"/>
+        <v>400</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>tekenbrief</t>
+        </is>
+      </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>QRA volgt</t>
+          <t>dolphins indicatief</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>LNG-zone (tanks + hervergassing)</t>
+          <t>LNG-envelop tot draaikom</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>36.3</v>
-      </c>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Invoer D51-D52</t>
-        </is>
-      </c>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>989</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>&gt;0</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr"/>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>3 tanks + optie 4e</t>
+          <t>vrij; QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Centrale + utilities (reservering)</t>
+          <t>LNG-tanks tot containerterrein</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>43.5</v>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>477</v>
       </c>
       <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>geen vast oppervlak</t>
-        </is>
-      </c>
+      <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>QRA volgt</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>STS-kranen F1 / F2 / F3</t>
+          <t>LNG-zone (tanks + hervergassing)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>6 / 12 / 20</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>6 / 12 / 20</t>
-        </is>
-      </c>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="D42" s="3" t="n"/>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Containers D19-F19</t>
+          <t>Invoer D51-D52</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>gelijk</t>
+          <t>3 tanks + optie 4e</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>TEU-grondslots stackzone F3 (28 m2/slot)</t>
+          <t>Centrale + utilities (reservering)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>slots</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="n">
-        <v>40558</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>40444</v>
-      </c>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="D43" s="3" t="n"/>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Containers F25</t>
+          <t>geen vast oppervlak</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>reservering</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Stackzone bruto</t>
+          <t>STS-kranen F1 / F2 / F3</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>113.6</v>
-      </c>
-      <c r="D44" s="3" t="n">
-        <v>113.2</v>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>6 / 12 / 20</t>
+        </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Containers F26</t>
+          <t>Containers D19-F19</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>gelijk</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Graansilo's 8 x D 30 m x 40 m</t>
+          <t>TEU-grondslots stackzone F3 (28 m2/slot)</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>169646</v>
+        <v>40558</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>154100</v>
+        <v>40444</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Overige terminals F9</t>
+          <t>Containers F25</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -1652,23 +1650,23 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>RoRo-parkeercapaciteit</t>
+          <t>Stackzone bruto</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>auto's</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>9698</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>113.6</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>7479</v>
+        <v>113.2</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Overige terminals F15</t>
+          <t>Containers F26</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -1680,117 +1678,137 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Centrale STEG-eenheden</t>
+          <t>Graansilo's 8 x D 30 m x 40 m</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>t</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2260</v>
+        <v>169646</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>2256</v>
+        <v>154100</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Overige terminals F30</t>
+          <t>Overige terminals F9</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>rekenvoorbeeld</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Havendiensten / sleepboten</t>
+          <t>RoRo-parkeercapaciteit</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="inlineStr"/>
+          <t>auto's</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>9698</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>7479</v>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F15</t>
+        </is>
+      </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>reservering</t>
+          <t>voldoet</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
+          <t>Centrale STEG-eenheden</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>334</v>
+        <v>2260</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="E49" s="3" t="inlineStr"/>
+        <v>2256</v>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Overige terminals F30</t>
+        </is>
+      </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>voldoet</t>
+          <t>rekenvoorbeeld</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 1</t>
+          <t>Havendiensten / sleepboten</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="n">
-        <v>1189081</v>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>43</v>
       </c>
       <c r="D50" s="3" t="n"/>
       <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>reservering</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
+          <t>Vrije breedte hoofdbekken met graanschip aan de kade</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1419486</v>
-      </c>
-      <c r="D51" s="3" t="n"/>
+        <v>334</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>220</v>
+      </c>
       <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>voldoet</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
+          <t>Binnenbekken gebaggerd fase 1</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1799,7 +1817,7 @@
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>1649890</v>
+        <v>1287977</v>
       </c>
       <c r="D52" s="3" t="n"/>
       <c r="E52" s="3" t="inlineStr"/>
@@ -1808,7 +1826,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Voorhaven + LNG-insteek gebaggerd</t>
+          <t>Binnenbekken gebaggerd fase 2 (cumulatief)</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1817,7 +1835,7 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>1132971</v>
+        <v>1510224</v>
       </c>
       <c r="D53" s="3" t="n"/>
       <c r="E53" s="3" t="inlineStr"/>
@@ -1826,7 +1844,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Havenbekken totaal (zone 1)</t>
+          <t>Binnenbekken gebaggerd fase 3 (cumulatief)</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1835,24 +1853,16 @@
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>2782861</v>
+        <v>1740629</v>
       </c>
       <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C6</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>ingevuld</t>
-        </is>
-      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Geul buiten de mond (zone 2 + 3)</t>
+          <t>Voorhaven + LNG-insteek gebaggerd</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1861,52 +1871,42 @@
         </is>
       </c>
       <c r="C55" s="4" t="n">
-        <v>7700000</v>
+        <v>1188749</v>
       </c>
       <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Grondwerk C7 + C8</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>gesplitst op -15 m</t>
-        </is>
-      </c>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Baggervolume zone 1 / 2 / 3</t>
+          <t>Havenbekken totaal (zone 1)</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>mln m3</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>59,1 / 29,9 / 3,6</t>
-        </is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>2929377</v>
       </c>
       <c r="D56" s="3" t="n"/>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Grondwerk F6-F8</t>
+          <t>Grondwerk C6</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>celmethode, indicatief</t>
+          <t>ingevuld</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+          <t>Geul buiten de mond (zone 2 + 3)</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1915,15 +1915,69 @@
         </is>
       </c>
       <c r="C57" s="4" t="n">
-        <v>3273444</v>
+        <v>4558615</v>
       </c>
       <c r="D57" s="3" t="n"/>
       <c r="E57" s="3" t="inlineStr">
         <is>
+          <t>Grondwerk C7 + C8</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>gesplitst op -15 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Baggervolume zone 1 / 2 / 3</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>mln m3</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>61,9 / 18,3 / 1,2</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n"/>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Grondwerk F6-F8</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>celmethode, indicatief</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Terreinophoging (terminals, LNG, centrale, havendienst)</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>3459480</v>
+      </c>
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
           <t>Grondwerk D21</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>ingevuld</t>
         </is>
@@ -1940,7 +1994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2137,26 +2191,26 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Eindpunt geul (voorlopig)</t>
+          <t>Eindpunt geul (natuurlijk -18,2 m)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>333795.61</v>
+        <v>312554.73</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7643823.84</v>
+        <v>7635252.11</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-21.2998354</v>
+        <v>-21.3751711</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-40.602281</v>
+        <v>-40.8079279</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>4303.4</v>
+        <v>2070.5</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>1515.5</v>
+        <v>1989.1</v>
       </c>
     </row>
     <row r="10">
@@ -2291,22 +2345,22 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>297643.11</v>
+        <v>297337.53</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7648245.24</v>
+        <v>7648101.61</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-21.2562317</v>
+        <v>-21.2574946</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-40.9501407</v>
+        <v>-40.9531014</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>832</v>
+        <v>799.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>456</v>
+        <v>464.8</v>
       </c>
     </row>
     <row r="15">
@@ -2351,22 +2405,22 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>295265.72</v>
+        <v>295137.77</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7649177.72</v>
+        <v>7648747.57</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-21.2475449</v>
+        <v>-21.2514147</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-40.9729295</v>
+        <v>-40.9742137</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>614.8</v>
+        <v>594.8</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>323.4</v>
+        <v>363.4</v>
       </c>
     </row>
     <row r="17">
@@ -2377,44 +2431,74 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Middelpunt draaikom binnenhaven</t>
+          <t>Middelpunt zwaaiplaats binnenhaven</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>295569.79</v>
+        <v>295561.07</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>7649774.96</v>
+        <v>7649824.37</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-21.242186</v>
+        <v>-21.2417388</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-40.969929</v>
+        <v>-40.970007</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>655</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DO overgetrokken van de Porto Central-render: schaal 10.035 m/px, draaiing 10.0 gr, render (812,5; 275) = A1.</t>
-        </is>
+        <v>265</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Begin bocht geul (R 3.400 m)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>301701.9</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>7648946.72</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>-21.250345</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>-40.9109605</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>1242.5</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>457.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E = 9.882546 x + 1.742559 y + 288626.228;  N = 1.742559 x + -9.882546 y + 7651301.871  (x, y = renderpixel, y omlaag).</t>
+          <t>DO overgetrokken van de Porto Central-render: schaal 10.035 m/px, draaiing 10.0 gr, render (812,5; 275) = A1.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t>E = 9.882546 x + 1.742559 y + 288626.228;  N = 1.742559 x + -9.882546 y + 7651301.871  (x, y = renderpixel, y omlaag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Lat/lon via pyproj (EPSG:31984 -&gt; EPSG:4326).</t>
         </is>
@@ -3526,7 +3610,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>DO: containerkade aan de westzijde van vinger 6, in het insteekbekken. Golftoets (DO-09): aan de oostzijde (voorhaven) wordt Hs 1,66 m (grens 0,5 m), in de insteek 0,01 m. Containerschepen varen met sleepboten door de draaikom (D 720 m) het hoofdbekken in, zwaaien op de zwaaiplaats binnenhaven (D 500 m = 1,5 LOA, met sleepboten; het hoofdbekken is daar verbreed) en worden achteruit de insteek in gesleept, zodat ze met de kop naar buiten afmeren. De zwaaiplaats ligt 165 m vrij van afgemeerde schepen en 91 m van de oever. Draaikom voorhaven 416 m vrij; stopweg 1.720 m = 5,1 LOA.</t>
+          <t>DO: containerkade aan de westzijde van vinger 6, in het insteekbekken. Golftoets (DO-09): aan de oostzijde (voorhaven) wordt Hs 2,08 m (grens 0,5 m), in de insteek 0,24 m. Containerschepen varen met sleepboten door de draaikom (D 720 m) het hoofdbekken in, zwaaien op de zwaaiplaats binnenhaven (D 670 m = 2 x LOA van het maatgevende containerschip; het hoofdbekken is daar verbreed, zodat de draai zonder krappe marges lukt) en worden achteruit de insteek in gesleept, zodat ze met de kop naar buiten afmeren. De zwaaiplaats ligt 115 m vrij van afgemeerde schepen en 156 m van de oever. Draaikom voorhaven 416 m vrij; stopweg 1.720 m = 5,1 LOA.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3558,7 +3642,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>DO: rechte geul 220 m, -18,20 m MLWS, in het verlengde van de havenmond; koppelpunt 1.500 m buiten de mond (A4). Bodemmodel uit GEBCO 2026 + Copernicus DEM (DO-10): het kustplateau is vlak (-13 tot -17 m); de natuurlijke bodem is pas op 35.000 m overal dieper dan -18,2 m MLWS (-15 m op 24.000 m). Geul daarom 35 km lang; zone 2/3 gesplitst op de -15 m-lijn.</t>
+          <t>DO: geul 220 m, -18,20 m MLWS: 2,5 km recht in het verlengde van de havenmond (koppelpunt sleepboten op 1.500 m, A4), dan een bocht met straal 3.400 m (ca. 10 x LOA, verbreed tot 260 m, A14) naar 145 gr en recht tot de natuurlijke -18,2 m MLWS. Bodemmodel GEBCO 2026 + Copernicus DEM (DO-10): naar het ZO is het veel eerder diep. Lengte buiten de mond 20,2 km met 19,5 mln m3 (rechtdoor: 35,0 km, 33,5 mln m3). De haven 1 km verder in zee leggen bespaart ca. 3,3 mln m3 bagger maar kost ca. 0,54 mln m3 extra stortsteen in de dammen: ongeveer kostenneutraal, daarom niet gedaan. Zone 2/3 gesplitst op de -15 m-lijn.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -3590,7 +3674,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>DO: LNG-steiger achter het midden van de zuidelijke dam (golftoets Hs 0,90 m &lt; 1,0 m; bij de havenmond 1,08 m). Tanks oostelijk in de LNG-zone: cryogene leiding ca. 1,4 km. Veiligheidszone 250 m rond schip/steiger en rond de tanks, nautische controlezone 500 m (Hong Kong LNG-terminal; literatuur 250-750 m): geen andere schepen of gebouwen in de 250 m-zones; draaikom 626 m buiten de zone, containerterrein 46 m buiten de tankzone. Ligplaats en vaarweg -16,20 m MLWS.</t>
+          <t>DO: LNG-steiger op de gunstigste plek achter de zuidelijke dam (golftoets met reflectie Hs 0,98 m &lt;= 1,0 m; bij de havenmond 1,98 m). Tanks in het zuidelijke deel van de LNG-zone, zodat de 250 m-zone ruim buiten het containerterrein blijft; cryogene leiding ca. 1,2 km. Veiligheidszone 250 m rond schip/steiger en rond de tanks, nautische controlezone 500 m (Hong Kong LNG-terminal; literatuur 250-750 m): geen andere schepen of gebouwen in de 250 m-zones; draaikom 739 m buiten de zone, containerterrein 227 m buiten de tankzone. Ligplaats en vaarweg -16,20 m MLWS.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3622,7 +3706,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>DO: graan 30,4 ha aan de noordkade (render 10) met silo en transportband; RoRo 30,2 ha in de noordoosthoek van vinger 7/8 met kade aan het insteekbekken; ieder een kade van 300 m en een eigen poort.</t>
+          <t>DO: graan 30,4 ha aan de noordkade (render 10) met silo en transportband; de graan- en havendienstkade zijn open kades op palen boven een golfdempend talud (Cr 0,45 i.p.v. 0,9 voor een kademuur; Hs 0,96 m). RoRo 30,2 ha op vinger 7/8 met kade 400 m dieper in de insteek (Hs 0,17 m &lt;= 0,3 m); ieder een kade van 300 m en een eigen poort.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -3654,7 +3738,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>DO: containers fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de westzijde van vinger 6; gebaggerd 118,9 / 141,9 / 165,0 ha; insteek zuid, hoofdbekken west en tweede insteek (122,1 ha) pas na 2045.</t>
+          <t>DO: containers fase 1 aan de noordkop (C1-C2), de kade groeit zuidwaarts langs de westzijde van vinger 6; gebaggerd 128,8 / 151,0 / 174,1 ha; insteek zuid, hoofdbekken west en tweede insteek (122,1 ha) pas na 2045.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -3782,7 +3866,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Celmethode (30 m) op het bodemmodel: zone 1 59,1, zone 2 29,9, zone 3 3,6 mln m3 (totaal 92,5 mln m3). Dieptezones per scheepstype (diepgang + 3,7 m): containers/graan -18,20, LNG -16,20, RoRo -13,70 m MLWS; besparing 0,75 mln m3. Ontwerpbodem per dieptezone als LandXML-oppervlak voor Civil 3D.</t>
+          <t>Celmethode (30 m) op het bodemmodel: zone 1 61,9, zone 2 18,3, zone 3 1,2 mln m3 (totaal 81,4 mln m3). Dieptezones per scheepstype (diepgang + 3,7 m): containers/graan -18,20, LNG -16,20, RoRo -13,70 m MLWS; besparing 0,86 mln m3. Ontwerpbodem per dieptezone als LandXML-oppervlak voor Civil 3D.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">

</xml_diff>